<commit_message>
fix: prevent duplicate memory edits and serialize memory writes
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -3744,12 +3744,12 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t xml:space="preserve">다른 기억을 기존 기억과 동일하게 수정</t>
+          <t xml:space="preserve">다른 기억을 기존 기억과 동일하게 수정; 다른 프로젝트 및 만료 기억과 동일한 내용으로 수정</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t xml:space="preserve">409, 중복 없음, 기존 revision 보존</t>
+          <t xml:space="preserve">409, 중복 없음, 기존 revision 보존; 다른 프로젝트/만료 기억은 충돌하지 않아 200</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -5769,31 +5769,58 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">검증 대기</t>
+          <t xml:space="preserve">BUG-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">기억 수정 중복 및 동시 저장</t>
+          <t xml:space="preserve">UT-050</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">이번 회귀 테스트에서 확인</t>
+          <t xml:space="preserve">동일 내용으로 수정해도 200; 활성 기억 중복 생성 / https://github.com/wjdwodhks35/Role-AI/actions/runs/38510187548</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">미수정</t>
+          <t xml:space="preserve">사용자·종류·프로젝트·내용 기준 활성 중복 확인 후 409; 변경 이력/버전 보존</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">미실행</t>
+          <t xml:space="preserve">전체 재검증 대기</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HARDEN-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-051</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">최초 동시 저장 테스트는 통과; 경쟁 가능성 예방 보강 / https://github.com/wjdwodhks35/Role-AI/actions/runs/38510187548</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SQLite BEGIN IMMEDIATE로 생성·추출·수정의 중복 확인과 쓰기 직렬화</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 재검증 대기</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:E3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add free local document retrieval with scoped sources and UI
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -46,7 +46,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">요구사항별 72개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">요구사항별 84개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -5362,8 +5362,872 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">73</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-073</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 업로드·내보내기·중복 제거</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">같은 내용의 파일명을 변경해 재등록하고 다른 프로젝트 등록</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">동일 범위는 동일 ID, 프로젝트별 분리, 원문 내보내기 일치</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_roundtrip_dedup_and_project</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">74</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-074</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 입력·경로·바이너리 제한</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">잘못된 경로/확장자/빈 내용/제어문자/16,001자 입력</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모두 422, 데이터 미저장</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_validation</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">75</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-075</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 인증·CSRF</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSRF 없이 저장, 로그인 없이 목록/저장</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403/401</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_auth_and_csrf</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">76</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-076</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 사용자 격리</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 계정으로 검색/조회/다운로드/삭제/대화 참조</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 사용자 데이터 미노출, 직접 ID 접근 404</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_user_isolation</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">77</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-077</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 프로젝트 검색·무근거·입력 제한</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">공통/프로젝트별 검색, 없는 키워드, 긴 검색어</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">범위 내 출처만 반환, 무근거 빈 목록, 길이초과422</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_search_scope_and_boundaries</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-078</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로컬 문서 대화·출처 이력</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ollama Mock 캡처, 명령이 포함된 문서 참조</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">비신뢰 데이터 구분, 출처 이력 저장, 도구없음, 기억 자동저장없음</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_prompt_and_history</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">79</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-079</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 대화 명시적 선택</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미선택/일치하지 않는 문서와 대화</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">참고자료 자동 전송없음, 검색근거 빈 목록</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_opt_in_and_no_match</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">80</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-080</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">유료/별도 엔진·프로젝트 차단</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OpenAI/OpenClaw/vLLM 또는 다른 프로젝트 문서 대화</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403/404, 메시지 미저장</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_chat_blocks_paid_gateway_and_wrong_project</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-081</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 문맥·선택 수 제한</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">긴 문서의 여러 검색결과, 6개 선택</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상위5개/JSON4500자 이하, 6개선택422</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_context_limits_and_selection</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-082</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 보관 한도·삭제 회수</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">32개 저장 후 추가/중복/삭제/재등록</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">추가409, 중복 허용, 발췌삭제 및 용량 회수</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_quota_and_cleanup</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">83</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-083</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 동시 중복 저장</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8개 동일 문서 병렬 등록</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">저장1개 및 동일ID</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_concurrent_duplicate</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">84</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-084</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">documents</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문서 삭제 후 이력·검색</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·테스트 계정·Mock 모델; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">대화 후 원문 삭제, 검색 및 대화 재조회</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">발췌검색없음, 식별자 이력 유지, 원문404</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_documents.py::test_document_deleted_source_history</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N73"/>
+  <autoFilter ref="A1:N85"/>
 </worksheet>
 </file>
 
@@ -5591,8 +6455,25 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-DOCUMENT-RAG 문서 보관·검색·출처·로컬 대화</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">txt/md 및 키워드 RAG, 유료 호출 차단</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 검증 대상</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
test: verify paid owner restrictions and document selection state
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -6305,17 +6305,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">의미검색·문서RAG·자동 보존정책</t>
+          <t xml:space="preserve">의미검색·PDF/DOCX·자동 보존정책</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">현재 키워드 검색만 제공</t>
+          <t xml:space="preserve">텍스트/Markdown 키워드 문서 RAG는 신규 구현; 의미 검색 등 후속</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">미구현</t>
+          <t xml:space="preserve">부분 구현</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add isolated PDF extraction and local semantic document retrieval
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -46,7 +46,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">요구사항별 84개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">95개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -6226,8 +6226,800 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">85</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-085</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF 추출·보관·검색·내보내기</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 PDF 생성 후 업로드/검색/추출텍스트 다운로드/재등록</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">페이지 표시 및 텍스트 추출, 검색 연결, 원본 미보관, 중복 제거</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_pdf_extract_store_search_export</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">86</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-086</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF 손상·암호화·스캔·범위 차단</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">손상/암호화/빈 페이지/21페이지/긴 추출문/경로 입력</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422 미저장, 스캔 OCR 필요 표시</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_pdf_rejects_unsupported_and_malformed</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-087</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF 전용 업로드 한도와 CSRF</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">512KiB 초과,64KiB 초과 유효PDF,CSRF 없는 업로드</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">초과413, 허용크기PDF는 파서 진행,CSRF403</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_pdf_body_limit_and_csrf</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">88</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-088</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF 격리 시간 및 플랫폼 오류</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">파서 timeout, Windows 직접실행 모사</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422/503, 정상처리로 가장하지 않음</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_pdf_parser_timeout_and_platform</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">89</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-089</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">벡터 기반 동의어 검색 경로</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">키워드가 없는 질의, Mock 로컬 임베딩으로 유사 문서 검색</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의미검색 순위 및 점수, 로컬embed/truncate=false/keepalive0</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_synonyms_without_keyword_match</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">90</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-090</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의미 검색 미설정·오류 구분</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모델 없음, 잘못된 반환 모델</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">503, 키워드 검색 독립 사용, 자동fallback 없음</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_disabled_and_no_hidden_fallback</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">91</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-091</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">잘못된 임베딩 벡터 차단</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">개수/차원/영벡터/불리언/범위/문자/타입 오류</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모두503</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_invalid_vectors</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">92</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-092</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원격·Cloud 임베딩 차단</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">remote_host 모델, 외부 Ollama URL</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">503, embed 미호출</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_remote_and_cloud_models_blocked</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-093</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의미 검색 접근권한 선검증</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">다른 프로젝트/사용자 ID, CSRF 미제공</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">404/403, 모델 호출 전 거절</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_user_project_and_csrf_before_inference</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">94</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-094</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">의미 검색 채팅·출처 이력</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로컬 Mock 임베딩과 모델 대화/기록 조회/유료 전송 시도</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">문맥 및 score 출처 저장, 유료 전송403</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_chat_context_history_and_paid_block</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">95</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-095</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pdf_semantic</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임베딩 장애·GPU 잠금</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 SQLite·pypdf 실제 추출·Mock 임베딩 HTTP; 유료 API·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로컬 타임아웃/협력 GPU 잠금 상태에서 의미검색</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">503, 대화 미저장, 자동fallback 없음</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_pdf_semantic.py::test_semantic_timeout_no_history_and_gpu_lock</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N85"/>
+  <autoFilter ref="A1:N96"/>
 </worksheet>
 </file>
 
@@ -6472,8 +7264,25 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-PDF-SEMANTIC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PDF 텍스트 추출/로컬 의미 검색/출처/UI</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동검증; 실제 임베딩 모델 품질 미검증, OCR/DOCX 미구현</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C14"/>
+  <autoFilter ref="A1:C15"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: archive 138 passing PDF and semantic retrieval tests
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -7097,17 +7097,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">의미검색·PDF/DOCX·자동 보존정책</t>
+          <t xml:space="preserve">DOCX·OCR·자동 보존정책</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">텍스트/Markdown 키워드 문서 RAG는 신규 구현; 의미 검색 등 후속</t>
+          <t xml:space="preserve">PDF·로컬 의미 검색은 추가; DOCX/OCR/자동 보존정책 후속</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">부분 구현</t>
+          <t xml:space="preserve">미구현 범위</t>
         </is>
       </c>
     </row>
@@ -7421,8 +7421,30 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">로컬 임베딩 모델 한국어 품질·GPU 메모리</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">설치된 로컬 임베딩 모델 및 실제 GPU</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add bounded AI-driven dataset collection schedules and local reviews
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -46,7 +46,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">95개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">104개 시나리오; 매개변수별 실행수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -7018,8 +7018,656 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">96</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-096</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 수집 계획 관리</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">주제·주기·횟수 등록 후 중지/재개/삭제</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">201 및 상태 저장·소유자 계획 관리</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_create_pause_resume_delete</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">97</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-097</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 수집 권한·네트워크·CSRF</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">비활성화 네트워크/CSRF없음/비소유자 접근</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403, 자동수집 시작 안함</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_owner_network_and_csrf</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">98</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-098</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 수집 주기·횟수 제한</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">빈 주제/0시간/31회 입력</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422, 무한 수집 정책 거절</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_input_limits</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">99</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-099</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">수집 계획 수량·소유권</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">계획5개 초과, 다른 사용자 조회/중지</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">409/404 및 타인 목록 미노출</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_plan_quota_and_foreign_access</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">100</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-100</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI 자동 탐색·파일·필드·샘플·로컬검수</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mock HF/Ollama로 실제 일정실행 및 정제·저장·조회</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30행 고정revision, 세역할Ollama검수, 사용자 승인 대기, 학습없음</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_autonomous_import_and_local_reviews</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">101</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-101</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">환각 후보·Cloud·불명 라이선스 차단</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미발견dataset/Cloud모델/unknown라이선스 선택</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실패기록, 다운로드/데이터셋/학습 없음</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_rejects_untrusted_candidates_and_license</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">102</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-102</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 검수 거절과 학습 분리</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Teacher가 reject 반환</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">후속검수 중단, 데이터 보관/미승인/학습없음</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_review_reject_no_training</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-103</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">예약 간격·중복 수집·중지</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">예약전 실행/다음실행 동일 파일/일정중지</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">예약전없음,중복skip,데이터1개,중지후실행없음</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_schedule_pause_and_dedup</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">104</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-104</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">collection</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">중단 Worker 복구·진행중 삭제 보호</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama·실제저장소; 유료 API/GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">running으로 남은 계획의 OS잠금 확보 및 복구</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실패이력/다음예약설정,진행중삭제409</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_collection.py::test_collection_interrupted_worker_recovery</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N96"/>
+  <autoFilter ref="A1:N105"/>
 </worksheet>
 </file>
 
@@ -7281,8 +7929,25 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-AUTO-COLLECTION</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AI 예약 수집·샘플 저장·무료검수·승인분리</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동테스트,실제HF/장기간/GPU대기</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C15"/>
+  <autoFilter ref="A1:C16"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: archive passing autonomous collection tests and worker guidance
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -8108,8 +8108,30 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 HF/Ollama 수집 및 장기간 예약 Worker</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 로컬모델·HF 설정·Worker 상시실행</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D7"/>
+  <autoFilter ref="A1:D8"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add scoped ChatGPT automatic learning approval policy
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -46,7 +46,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">104개 시나리오; 매개변수별 실행수는 결과에 기록</t>
+          <t xml:space="preserve">117개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -7666,8 +7666,944 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">105</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-105</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ChatGPT 자동 승인 기본 꺼짐</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정책 조회 및 꺼진 상태에서 심사</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">꺼짐/수동큐/승인409, 유료 호출 없음</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_policy_default_off_and_scope</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">106</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-106</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 위임·유료 동의·설정·학습 한도</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미동의/권리확인없음/101step/미설정OpenAI 활성화</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422/503, API 미호출</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_policy_requires_consent_and_configuration</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">107</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-107</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 승인 정책 권한·사용자 격리</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSRF 없음/비소유자/다른 데이터 ID 심사</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403/404, 타인 감사이력 미노출</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_policy_owner_and_csrf</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">108</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-108</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPT 전체 선택 데이터 승인·기록</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정책 켠 후 실제Responses형 Mock심사</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습·평가30개 전송, 승인해시/역할/한도/GPT검수 저장, 학습 미시작</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_gpt_full_selected_data_approval_no_training</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">109</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-109</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPT 거절·위험·응답·연결 오류</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reject/risks/bad JSON/timeout 응답</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미승인, 감사이력, 동일심사 재호출409</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_gpt_reject_risk_and_failures_no_approval</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">110</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-110</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 GPT 예산 선확인</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">낮은 요청예산으로 심사</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">failed, 실제 API 요청없음</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_approval_budget_checked_before_request</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">111</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-111</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">심사 중 위임 철회·데이터 변경</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPT응답 전 모드끄기/데이터revision변경</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cancelled, 승인없음</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_approval_race_revocation_and_data_revision</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">112</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-112</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">모델·비용 정책 바인딩</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">등록 후 일일예산/모델파일 변경</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">409, 기존 위임으로 API 미호출</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_policy_model_and_budget_change_blocked</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">113</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-113</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 위임 끄기와 대기 작업 철회</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동승인후 수동큐등록, 모드끄기</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">승인해시제거, 대기작업취소, 감사revoked</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_policy_disable_revokes_queued_approval</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">114</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-114</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">동시 GPT 승인 요청 중복 결제 방지</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">같은데이터에2개병렬심사</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">하나200/하나409, API1회</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_approval_concurrent_request_single_paid_call</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">115</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-115</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">수집 Worker 자동 위임 통합</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HF/로컬Mock수집 후 활성정책의 GPT심사</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 승인 적용, 학습/배포 미시작</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_collection_invokes_enabled_gpt_policy</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">116</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-116</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">위임 범위와 로컬검수 제한</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">수동데이터/31행/Teacher거절</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">409, API미호출</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_approval_scope_and_local_review_blocks</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">117</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-117</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">auto_approval</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">변경된 데이터 파일 자동 승인 차단</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·Mock HF/Ollama/OpenAI·가짜Weights; 실제 결제/GPU 없음</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">압축샘플파일을심사전변조</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">409, API미호출</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_auto_approval.py::test_auto_approval_tampered_artifact_blocked</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N105"/>
+  <autoFilter ref="A1:N118"/>
 </worksheet>
 </file>
 
@@ -7946,8 +8882,25 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPT-AUTO-APPROVAL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">소유자옵트인/전체선택샘플GPT심사/승인/철회/감사/수집연동</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mock자동테스트,실제유료/GPU대기</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C16"/>
+  <autoFilter ref="A1:C17"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs: archive 173 passing GPT automatic approval policy tests
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -9083,8 +9083,30 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPT 자동 심사·청구·GPU 학습 정책 연동</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OpenAI 키/비용 동의/로컬학습 모델/Worker</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D8"/>
+  <autoFilter ref="A1:D9"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: add configurable GPU memory budgets and training allocator limits
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -46,7 +46,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">117개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t xml:space="preserve">129개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -8602,8 +8602,872 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">118</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-118</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPU 설정 저장·측정·재시작 지속</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">소유자가 한도 저장 후 별도 Settings로 읽기/상태조회</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원자적 저장, 실제측정형식/유효한도, 전역강제상한아님표시</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_settings_persistence_and_measurement</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">119</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-119</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPU 설정 범위·자료형 검증</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">511MiB/음수여유/0예상값/불리언/소수MiB 입력</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422, 설정 파일 미작성</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_settings_validation</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">120</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-120</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPU 설정 권한·CSRF</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSRF없는 저장/일반회원 조회·변경</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">403</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_settings_owner_and_csrf</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">121</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-121</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VRAM 한도 경계·물리 용량·여유</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">사용+예상=한도 및 1MiB초과, 큰설정/과도한여유</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">경계허용, 초과차단, 실제총량-여유로제한</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_admission_exact_boundary_and_physical_clamp</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">122</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-122</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미측정·꺼짐·설정손상·복구</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">측정불가/검사off/on/손상파일/재저장</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">off계속가능,on차단,손상표시와저장복구</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_unavailable_disabled_and_corrupt_repair</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">123</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-123</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NVIDIA 측정 안전한 실행·검증</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CSV정상/N-A/timeout 가짜명령 실행</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GPU0고정·shell없음·3초한도·이상값차단</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_nvidia_smi_parsing_and_timeout</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">124</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-124</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ollama 작업 전 VRAM 검사·반납</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">메모리초과/허용상태 채팅/정책끄기</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">초과503 API/메시지없음, 허용keepalive0,off기존5m</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_ollama_block_and_release_after_allowed_request</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">125</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-125</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임베딩·OpenClaw 예산 검사</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">상한초과 상태 의미검색/Gateway 호출</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">503/ProviderUnavailable, 모델API호출없음</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_semantic_and_gateway_preflight</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">126</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-126</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원격GPU 오적용 차단·Mock 제외</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원격Ollama 한도검사, 측정불가Mock채팅</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">원격차단, Mock200</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_remote_ollama_rejected_and_mock_exempt</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">127</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-127</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습 할당기 VRAM 예산</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8GiB장치에5GiB할당범위/검사off/총량0</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fraction0.625 GPU0, off무설정, 총량불명차단</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_training_allocator_fraction</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">128</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-128</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습 VRAM초과·승인보존</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">승인/큐등록 후 예산초과 Worker 실행</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blocked, Trainer 미실행, 승인해시 유지</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_training_blocked_keeps_approval</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">129</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-129</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gpu_resources</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습 CUDA OOM 대기 전환</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시SQLite·FakeGPU/명령/할당기·MockHTTP; 실제GPU/유료없음</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TorchOOM 모사</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ResourcesBusy로 전환, 실제GPU사용없음</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_gpu_resources.py::test_gpu_training_oom_becomes_resource_wait</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N118"/>
+  <autoFilter ref="A1:N130"/>
 </worksheet>
 </file>
 
@@ -8899,8 +9763,25 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-GPU-BUDGET</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">최대VRAM/여유/작업예산/모니터링/학습할당기/대기</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동테스트,실제4060Ti/WSL/컨테이너대기</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C17"/>
+  <autoFilter ref="A1:C18"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: disable inherited collector HTTP healthcheck and archive GPU tests
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -9986,8 +9986,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU VRAM 측정·작업예산·할당기·DockerGPU0</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4060Ti/드라이버/WSL/Toolkit/실제PyTorch훈련</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: full selected-sample review, fixed benchmarks and model candidate lifecycle
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -9466,8 +9466,944 @@
         </is>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">130</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-130</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 학습·평가 샘플 검수</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_covers_train_and_eval</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">131</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-131</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">거부·위험·비정상응답 차단</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_full_review_rejects_or_fails_closed</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">132</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-132</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">검수 중 오류 부분 통과 방지</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_review_error_does_not_store_partial_pass</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">133</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-133</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">기존 3개 검수 재승인 차단</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_old_preview_cannot_approve</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">134</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-134</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">고정 평가·승인 해시 연결</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_registration_and_immutable_plan</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">135</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-135</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">평가 입력 제한·중복</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_limits_and_duplicates</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">136</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-136</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">학습 문항 유출·미등록 평가 차단</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_leakage_and_unknown_suite</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">137</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-137</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">정답 정규화·응답 검증</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_benchmark_exact_match_and_response_validation</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">138</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-138</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">통합 상태·가짜 진행률 방지</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_dashboard_no_worker_or_percent_claim</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">139</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-139</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">후보 선택·롤백·동시 변경</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_selection_rollback_and_cas</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">140</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-140</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">변조·퇴행·평가누락·가짜학습 차단</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_candidate_validation_blocks_bad_versions</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">141</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-141</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">롤백 이전 파일 재검증</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_rollback_revalidates_previous_files</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">142</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UT-142</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REQ-QUALITY-LIFECYCLE</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">quality_lifecycle</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">API·단위/흐름</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">소유자·CSRF 제한</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 GPU·유료 API 미사용; 파일과 모델 응답은 테스트용</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">임시 DB·합성 샘플·모사 모델로 성공·실패 및 저장 상태 확인</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·고정 평가·후보 검증·접근 제어 기준 충족</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tests/test_quality_lifecycle.py::test_lifecycle_owner_and_csrf</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N130"/>
+  <autoFilter ref="A1:N143"/>
 </worksheet>
 </file>
 
@@ -9780,8 +10716,25 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체검수·고정평가·배포후보·통합현황</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">행별 로컬검수/학습계획 평가 고정/파일 검증/후보 롤백/권한</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">자동 검증; 실제 GPU 생성·배포는 별도</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C18"/>
+  <autoFilter ref="A1:C19"/>
 </worksheet>
 </file>
 
@@ -10008,8 +10961,30 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ENV-QUALITY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">전체 검수·GPU 전후 고정 질문 생성</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">실제 Ollama 및 기반 모델·GPU</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D11"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat: preview request analysis and explicitly apply suggested chat roles
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="단위테스트" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="요구사항커버리지" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="실환경검증" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="결함이력" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="단위테스트" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항커버리지" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실환경검증" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결함이력" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N172"/>
+  <dimension ref="A1:N180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9825,9 +9825,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L163" t="inlineStr"/>
-      <c r="M163" t="inlineStr"/>
-      <c r="N163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -9885,9 +9882,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L164" t="inlineStr"/>
-      <c r="M164" t="inlineStr"/>
-      <c r="N164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -9945,9 +9939,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L165" t="inlineStr"/>
-      <c r="M165" t="inlineStr"/>
-      <c r="N165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10005,9 +9996,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L166" t="inlineStr"/>
-      <c r="M166" t="inlineStr"/>
-      <c r="N166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -10065,9 +10053,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L167" t="inlineStr"/>
-      <c r="M167" t="inlineStr"/>
-      <c r="N167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -10125,9 +10110,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="inlineStr"/>
-      <c r="N168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -10185,9 +10167,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L169" t="inlineStr"/>
-      <c r="M169" t="inlineStr"/>
-      <c r="N169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -10245,9 +10224,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L170" t="inlineStr"/>
-      <c r="M170" t="inlineStr"/>
-      <c r="N170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -10305,9 +10281,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L171" t="inlineStr"/>
-      <c r="M171" t="inlineStr"/>
-      <c r="N171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -10365,12 +10338,489 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L172" t="inlineStr"/>
-      <c r="M172" t="inlineStr"/>
-      <c r="N172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>172</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>UT-172</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>test_preview_only_suggests_roles_without_writes</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_only_suggests_roles_without_writes</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr"/>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>173</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>UT-173</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>test_preview_rejects_cloud_failures_and_bad_schema</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_rejects_cloud_failures_and_bad_schema</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr"/>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>174</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>UT-174</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>test_preview_validates_input_before_call</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_validates_input_before_call</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr"/>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>175</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>UT-175</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>test_preview_requires_local_model_endpoint</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_requires_local_model_endpoint</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr"/>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>176</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>UT-176</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>test_preview_auth_csrf_and_owner_guards</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_auth_csrf_and_owner_guards</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr"/>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>177</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>UT-177</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>test_preview_timeout_and_lock_release</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_timeout_and_lock_release</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr"/>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>UT-178</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>test_recommendation_deduplicates_and_does_not_dispatch</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_recommendation_deduplicates_and_does_not_dispatch</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr"/>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>179</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>UT-179</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>REQ-REQUEST-ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>요구사항 분석 미리보기</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>test_preview_rejects_parallel_requests</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>합성 요청과 격리 DB</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>입력·권한·모델 응답 조건별 API 호출</t>
+        </is>
+      </c>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>참고 분석만 반환, 작업 미실행</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>tests/test_request_analysis.py::test_preview_rejects_parallel_requests</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr"/>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N172"/>
+  <autoFilter ref="A1:N180"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add privacy-preserving local readiness and opt-in Ollama checks
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N180"/>
+  <dimension ref="A1:N191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10819,8 +10819,426 @@
       <c r="M180" t="inlineStr"/>
       <c r="N180" t="inlineStr"/>
     </row>
+    <row r="181">
+      <c r="A181" t="str">
+        <v>180</v>
+      </c>
+      <c r="B181" t="str">
+        <v>UT-180</v>
+      </c>
+      <c r="C181" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D181" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E181" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F181" t="str">
+        <v>test_inventory_never_reads_settings_or_database</v>
+      </c>
+      <c r="G181" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H181" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I181" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J181" t="str">
+        <v>tests/test_preflight.py::test_inventory_never_reads_settings_or_database</v>
+      </c>
+      <c r="K181" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L181"/>
+      <c r="M181"/>
+      <c r="N181"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="str">
+        <v>181</v>
+      </c>
+      <c r="B182" t="str">
+        <v>UT-181</v>
+      </c>
+      <c r="C182" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D182" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E182" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F182" t="str">
+        <v>test_inventory_missing_paths_creates_nothing</v>
+      </c>
+      <c r="G182" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H182" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I182" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J182" t="str">
+        <v>tests/test_preflight.py::test_inventory_missing_paths_creates_nothing</v>
+      </c>
+      <c r="K182" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L182"/>
+      <c r="M182"/>
+      <c r="N182"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="str">
+        <v>182</v>
+      </c>
+      <c r="B183" t="str">
+        <v>UT-182</v>
+      </c>
+      <c r="C183" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D183" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E183" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F183" t="str">
+        <v>test_inventory_parses_whitelisted_fields_only</v>
+      </c>
+      <c r="G183" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H183" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I183" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J183" t="str">
+        <v>tests/test_preflight.py::test_inventory_parses_whitelisted_fields_only</v>
+      </c>
+      <c r="K183" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L183"/>
+      <c r="M183"/>
+      <c r="N183"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="str">
+        <v>183</v>
+      </c>
+      <c r="B184" t="str">
+        <v>UT-183</v>
+      </c>
+      <c r="C184" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D184" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E184" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F184" t="str">
+        <v>test_symlink_metadata_does_not_follow_target</v>
+      </c>
+      <c r="G184" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H184" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I184" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J184" t="str">
+        <v>tests/test_preflight.py::test_symlink_metadata_does_not_follow_target</v>
+      </c>
+      <c r="K184" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L184"/>
+      <c r="M184"/>
+      <c r="N184"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="str">
+        <v>184</v>
+      </c>
+      <c r="B185" t="str">
+        <v>UT-184</v>
+      </c>
+      <c r="C185" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D185" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E185" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F185" t="str">
+        <v>test_remote_or_credential_urls_are_rejected</v>
+      </c>
+      <c r="G185" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H185" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I185" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J185" t="str">
+        <v>tests/test_preflight.py::test_remote_or_credential_urls_are_rejected</v>
+      </c>
+      <c r="K185" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L185"/>
+      <c r="M185"/>
+      <c r="N185"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="str">
+        <v>185</v>
+      </c>
+      <c r="B186" t="str">
+        <v>UT-185</v>
+      </c>
+      <c r="C186" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D186" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E186" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F186" t="str">
+        <v>test_metadata_checks_never_generate</v>
+      </c>
+      <c r="G186" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H186" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I186" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J186" t="str">
+        <v>tests/test_preflight.py::test_metadata_checks_never_generate</v>
+      </c>
+      <c r="K186" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L186"/>
+      <c r="M186"/>
+      <c r="N186"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="str">
+        <v>186</v>
+      </c>
+      <c r="B187" t="str">
+        <v>UT-186</v>
+      </c>
+      <c r="C187" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D187" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E187" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F187" t="str">
+        <v>test_inference_is_explicit_bounded_local_and_sanitized</v>
+      </c>
+      <c r="G187" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H187" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I187" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J187" t="str">
+        <v>tests/test_preflight.py::test_inference_is_explicit_bounded_local_and_sanitized</v>
+      </c>
+      <c r="K187" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L187"/>
+      <c r="M187"/>
+      <c r="N187"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="str">
+        <v>187</v>
+      </c>
+      <c r="B188" t="str">
+        <v>UT-187</v>
+      </c>
+      <c r="C188" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D188" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E188" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F188" t="str">
+        <v>test_bad_cli_options_fail_without_inventory</v>
+      </c>
+      <c r="G188" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H188" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I188" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J188" t="str">
+        <v>tests/test_preflight.py::test_bad_cli_options_fail_without_inventory</v>
+      </c>
+      <c r="K188" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L188"/>
+      <c r="M188"/>
+      <c r="N188"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="str">
+        <v>188</v>
+      </c>
+      <c r="B189" t="str">
+        <v>UT-188</v>
+      </c>
+      <c r="C189" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D189" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E189" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F189" t="str">
+        <v>test_command_errors_are_sanitized</v>
+      </c>
+      <c r="G189" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H189" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I189" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J189" t="str">
+        <v>tests/test_preflight.py::test_command_errors_are_sanitized</v>
+      </c>
+      <c r="K189" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L189"/>
+      <c r="M189"/>
+      <c r="N189"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="str">
+        <v>189</v>
+      </c>
+      <c r="B190" t="str">
+        <v>UT-189</v>
+      </c>
+      <c r="C190" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D190" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E190" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F190" t="str">
+        <v>test_remote_docker_context_is_not_reported_as_local</v>
+      </c>
+      <c r="G190" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H190" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I190" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J190" t="str">
+        <v>tests/test_preflight.py::test_remote_docker_context_is_not_reported_as_local</v>
+      </c>
+      <c r="K190" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L190"/>
+      <c r="M190"/>
+      <c r="N190"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="str">
+        <v>190</v>
+      </c>
+      <c r="B191" t="str">
+        <v>UT-190</v>
+      </c>
+      <c r="C191" t="str">
+        <v>REQ-PREFLIGHT</v>
+      </c>
+      <c r="D191" t="str">
+        <v>로컬 준비 상태 진단</v>
+      </c>
+      <c r="E191" t="str">
+        <v>단위/CLI</v>
+      </c>
+      <c r="F191" t="str">
+        <v>test_docker_host_override_is_not_contacted</v>
+      </c>
+      <c r="G191" t="str">
+        <v>격리 임시 디렉터리·가짜 서비스</v>
+      </c>
+      <c r="H191" t="str">
+        <v>상태·URL·네트워크 조건별 진단</v>
+      </c>
+      <c r="I191" t="str">
+        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
+      </c>
+      <c r="J191" t="str">
+        <v>tests/test_preflight.py::test_docker_host_override_is_not_contacted</v>
+      </c>
+      <c r="K191" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L191"/>
+      <c r="M191"/>
+      <c r="N191"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N180"/>
+  <autoFilter ref="A1:N191"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add pinned local AI judge and approved on-policy RLAIF GRPO training
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N191"/>
+  <dimension ref="A1:N211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11237,8 +11237,768 @@
       <c r="M191"/>
       <c r="N191"/>
     </row>
+    <row r="192">
+      <c r="A192" t="str">
+        <v>191</v>
+      </c>
+      <c r="B192" t="str">
+        <v>UT-191</v>
+      </c>
+      <c r="C192" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D192" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E192" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F192" t="str">
+        <v>test_judge_feedback_strict_schema</v>
+      </c>
+      <c r="G192" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H192" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I192" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J192" t="str">
+        <v>tests/test_ai_judge.py::test_judge_feedback_strict_schema</v>
+      </c>
+      <c r="K192" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L192"/>
+      <c r="M192"/>
+      <c r="N192"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="str">
+        <v>192</v>
+      </c>
+      <c r="B193" t="str">
+        <v>UT-192</v>
+      </c>
+      <c r="C193" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D193" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E193" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F193" t="str">
+        <v>test_reward_weighting_uncertainty_and_zero_constraints</v>
+      </c>
+      <c r="G193" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H193" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I193" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J193" t="str">
+        <v>tests/test_ai_judge.py::test_reward_weighting_uncertainty_and_zero_constraints</v>
+      </c>
+      <c r="K193" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L193"/>
+      <c r="M193"/>
+      <c r="N193"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="str">
+        <v>193</v>
+      </c>
+      <c r="B194" t="str">
+        <v>UT-193</v>
+      </c>
+      <c r="C194" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D194" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E194" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F194" t="str">
+        <v>test_judge_failures_never_become_zero_rewards</v>
+      </c>
+      <c r="G194" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H194" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I194" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J194" t="str">
+        <v>tests/test_ai_judge.py::test_judge_failures_never_become_zero_rewards</v>
+      </c>
+      <c r="K194" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L194"/>
+      <c r="M194"/>
+      <c r="N194"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="str">
+        <v>194</v>
+      </c>
+      <c r="B195" t="str">
+        <v>UT-194</v>
+      </c>
+      <c r="C195" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D195" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E195" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F195" t="str">
+        <v>test_pinning_calibration_and_budget</v>
+      </c>
+      <c r="G195" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H195" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I195" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J195" t="str">
+        <v>tests/test_ai_judge.py::test_pinning_calibration_and_budget</v>
+      </c>
+      <c r="K195" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L195"/>
+      <c r="M195"/>
+      <c r="N195"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="str">
+        <v>195</v>
+      </c>
+      <c r="B196" t="str">
+        <v>UT-195</v>
+      </c>
+      <c r="C196" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D196" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E196" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F196" t="str">
+        <v>test_judge_local_endpoint_only</v>
+      </c>
+      <c r="G196" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H196" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I196" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J196" t="str">
+        <v>tests/test_ai_judge.py::test_judge_local_endpoint_only</v>
+      </c>
+      <c r="K196" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L196"/>
+      <c r="M196"/>
+      <c r="N196"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="str">
+        <v>196</v>
+      </c>
+      <c r="B197" t="str">
+        <v>UT-196</v>
+      </c>
+      <c r="C197" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D197" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E197" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F197" t="str">
+        <v>test_judge_disabled_and_deadline_guards</v>
+      </c>
+      <c r="G197" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H197" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I197" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J197" t="str">
+        <v>tests/test_ai_judge.py::test_judge_disabled_and_deadline_guards</v>
+      </c>
+      <c r="K197" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L197"/>
+      <c r="M197"/>
+      <c r="N197"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="str">
+        <v>197</v>
+      </c>
+      <c r="B198" t="str">
+        <v>UT-197</v>
+      </c>
+      <c r="C198" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D198" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E198" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F198" t="str">
+        <v>test_reward_recorder_preserves_exact_rollouts_and_step</v>
+      </c>
+      <c r="G198" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H198" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I198" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J198" t="str">
+        <v>tests/test_ai_judge.py::test_reward_recorder_preserves_exact_rollouts_and_step</v>
+      </c>
+      <c r="K198" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L198"/>
+      <c r="M198"/>
+      <c r="N198"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="str">
+        <v>198</v>
+      </c>
+      <c r="B199" t="str">
+        <v>UT-198</v>
+      </c>
+      <c r="C199" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D199" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E199" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F199" t="str">
+        <v>test_recorder_failure_does_not_write_fabricated_reward</v>
+      </c>
+      <c r="G199" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H199" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I199" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J199" t="str">
+        <v>tests/test_ai_judge.py::test_recorder_failure_does_not_write_fabricated_reward</v>
+      </c>
+      <c r="K199" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L199"/>
+      <c r="M199"/>
+      <c r="N199"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="str">
+        <v>199</v>
+      </c>
+      <c r="B200" t="str">
+        <v>UT-199</v>
+      </c>
+      <c r="C200" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D200" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E200" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F200" t="str">
+        <v>test_rlaif_approval_without_paid_orchestrator</v>
+      </c>
+      <c r="G200" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H200" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I200" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J200" t="str">
+        <v>tests/test_rlaif.py::test_rlaif_approval_without_paid_orchestrator</v>
+      </c>
+      <c r="K200" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L200"/>
+      <c r="M200"/>
+      <c r="N200"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="str">
+        <v>200</v>
+      </c>
+      <c r="B201" t="str">
+        <v>UT-200</v>
+      </c>
+      <c r="C201" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D201" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E201" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F201" t="str">
+        <v>test_rlaif_plan_gates</v>
+      </c>
+      <c r="G201" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H201" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I201" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J201" t="str">
+        <v>tests/test_rlaif.py::test_rlaif_plan_gates</v>
+      </c>
+      <c r="K201" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L201"/>
+      <c r="M201"/>
+      <c r="N201"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="str">
+        <v>201</v>
+      </c>
+      <c r="B202" t="str">
+        <v>UT-201</v>
+      </c>
+      <c r="C202" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D202" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E202" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F202" t="str">
+        <v>test_disabled_rlaif_does_not_reuse_sft_permission</v>
+      </c>
+      <c r="G202" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H202" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I202" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J202" t="str">
+        <v>tests/test_rlaif.py::test_disabled_rlaif_does_not_reuse_sft_permission</v>
+      </c>
+      <c r="K202" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L202"/>
+      <c r="M202"/>
+      <c r="N202"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="str">
+        <v>202</v>
+      </c>
+      <c r="B203" t="str">
+        <v>UT-202</v>
+      </c>
+      <c r="C203" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D203" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E203" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F203" t="str">
+        <v>test_failed_calibration_preserves_previous_approval</v>
+      </c>
+      <c r="G203" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H203" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I203" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J203" t="str">
+        <v>tests/test_rlaif.py::test_failed_calibration_preserves_previous_approval</v>
+      </c>
+      <c r="K203" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L203"/>
+      <c r="M203"/>
+      <c r="N203"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="str">
+        <v>203</v>
+      </c>
+      <c r="B204" t="str">
+        <v>UT-203</v>
+      </c>
+      <c r="C204" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D204" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E204" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F204" t="str">
+        <v>test_worker_dispatches_current_policy_training_without_activation</v>
+      </c>
+      <c r="G204" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H204" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I204" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J204" t="str">
+        <v>tests/test_rlaif.py::test_worker_dispatches_current_policy_training_without_activation</v>
+      </c>
+      <c r="K204" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L204"/>
+      <c r="M204"/>
+      <c r="N204"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="str">
+        <v>204</v>
+      </c>
+      <c r="B205" t="str">
+        <v>UT-204</v>
+      </c>
+      <c r="C205" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D205" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E205" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F205" t="str">
+        <v>test_worker_rejects_revoked_rlaif_before_training</v>
+      </c>
+      <c r="G205" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H205" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I205" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J205" t="str">
+        <v>tests/test_rlaif.py::test_worker_rejects_revoked_rlaif_before_training</v>
+      </c>
+      <c r="K205" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L205"/>
+      <c r="M205"/>
+      <c r="N205"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="str">
+        <v>205</v>
+      </c>
+      <c r="B206" t="str">
+        <v>UT-205</v>
+      </c>
+      <c r="C206" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D206" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E206" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F206" t="str">
+        <v>test_parent_sft_adapter_is_pinned_and_revalidated</v>
+      </c>
+      <c r="G206" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H206" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I206" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J206" t="str">
+        <v>tests/test_rlaif.py::test_parent_sft_adapter_is_pinned_and_revalidated</v>
+      </c>
+      <c r="K206" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L206"/>
+      <c r="M206"/>
+      <c r="N206"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="str">
+        <v>206</v>
+      </c>
+      <c r="B207" t="str">
+        <v>UT-206</v>
+      </c>
+      <c r="C207" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D207" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E207" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F207" t="str">
+        <v>test_preview_requires_consent_owner_and_does_not_enqueue</v>
+      </c>
+      <c r="G207" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H207" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I207" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J207" t="str">
+        <v>tests/test_rlaif.py::test_preview_requires_consent_owner_and_does_not_enqueue</v>
+      </c>
+      <c r="K207" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L207"/>
+      <c r="M207"/>
+      <c r="N207"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="str">
+        <v>207</v>
+      </c>
+      <c r="B208" t="str">
+        <v>UT-207</v>
+      </c>
+      <c r="C208" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D208" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E208" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F208" t="str">
+        <v>test_candidate_rejects_unqualified_rlaif</v>
+      </c>
+      <c r="G208" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H208" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I208" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J208" t="str">
+        <v>tests/test_rlaif.py::test_candidate_rejects_unqualified_rlaif</v>
+      </c>
+      <c r="K208" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L208"/>
+      <c r="M208"/>
+      <c r="N208"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="str">
+        <v>208</v>
+      </c>
+      <c r="B209" t="str">
+        <v>UT-208</v>
+      </c>
+      <c r="C209" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D209" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E209" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F209" t="str">
+        <v>test_reward_history_is_owner_bound_and_hash_checked</v>
+      </c>
+      <c r="G209" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H209" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I209" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J209" t="str">
+        <v>tests/test_rlaif.py::test_reward_history_is_owner_bound_and_hash_checked</v>
+      </c>
+      <c r="K209" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L209"/>
+      <c r="M209"/>
+      <c r="N209"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="str">
+        <v>209</v>
+      </c>
+      <c r="B210" t="str">
+        <v>UT-209</v>
+      </c>
+      <c r="C210" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D210" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E210" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F210" t="str">
+        <v>test_grpo_generation_settings_and_long_prompt_rejection</v>
+      </c>
+      <c r="G210" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H210" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I210" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J210" t="str">
+        <v>tests/test_rlaif.py::test_grpo_generation_settings_and_long_prompt_rejection</v>
+      </c>
+      <c r="K210" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L210"/>
+      <c r="M210"/>
+      <c r="N210"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="str">
+        <v>210</v>
+      </c>
+      <c r="B211" t="str">
+        <v>UT-210</v>
+      </c>
+      <c r="C211" t="str">
+        <v>REQ-RLAIF</v>
+      </c>
+      <c r="D211" t="str">
+        <v>AI 피드백 강화학습</v>
+      </c>
+      <c r="E211" t="str">
+        <v>단위/API</v>
+      </c>
+      <c r="F211" t="str">
+        <v>test_resource_retry_preserves_partial_attempt</v>
+      </c>
+      <c r="G211" t="str">
+        <v>합성 평가·격리 데이터</v>
+      </c>
+      <c r="H211" t="str">
+        <v>정책·보상·승인·작업·후보 조건 검사</v>
+      </c>
+      <c r="I211" t="str">
+        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
+      </c>
+      <c r="J211" t="str">
+        <v>tests/test_rlaif.py::test_resource_retry_preserves_partial_attempt</v>
+      </c>
+      <c r="K211" t="str">
+        <v>미실행</v>
+      </c>
+      <c r="L211"/>
+      <c r="M211"/>
+      <c r="N211"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N191"/>
+  <autoFilter ref="A1:N211"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
test: register foundation scenarios in the ordered QA plan
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="단위테스트" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항커버리지" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="실환경검증" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="결함이력" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="요약" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="단위테스트" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="요구사항커버리지" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="실환경검증" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="결함이력" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$229</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>142개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>228개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N211"/>
+  <dimension ref="A1:N229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10395,9 +10395,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L173" t="inlineStr"/>
-      <c r="M173" t="inlineStr"/>
-      <c r="N173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10455,9 +10452,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L174" t="inlineStr"/>
-      <c r="M174" t="inlineStr"/>
-      <c r="N174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -10515,9 +10509,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L175" t="inlineStr"/>
-      <c r="M175" t="inlineStr"/>
-      <c r="N175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -10575,9 +10566,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L176" t="inlineStr"/>
-      <c r="M176" t="inlineStr"/>
-      <c r="N176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -10635,9 +10623,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L177" t="inlineStr"/>
-      <c r="M177" t="inlineStr"/>
-      <c r="N177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10695,9 +10680,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L178" t="inlineStr"/>
-      <c r="M178" t="inlineStr"/>
-      <c r="N178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -10755,9 +10737,6 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L179" t="inlineStr"/>
-      <c r="M179" t="inlineStr"/>
-      <c r="N179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -10815,1190 +10794,2802 @@
           <t>미실행</t>
         </is>
       </c>
-      <c r="L180" t="inlineStr"/>
-      <c r="M180" t="inlineStr"/>
-      <c r="N180" t="inlineStr"/>
     </row>
     <row r="181">
-      <c r="A181" t="str">
-        <v>180</v>
-      </c>
-      <c r="B181" t="str">
-        <v>UT-180</v>
-      </c>
-      <c r="C181" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D181" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E181" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F181" t="str">
-        <v>test_inventory_never_reads_settings_or_database</v>
-      </c>
-      <c r="G181" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H181" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I181" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J181" t="str">
-        <v>tests/test_preflight.py::test_inventory_never_reads_settings_or_database</v>
-      </c>
-      <c r="K181" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L181"/>
-      <c r="M181"/>
-      <c r="N181"/>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>180</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>UT-180</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>test_inventory_never_reads_settings_or_database</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_inventory_never_reads_settings_or_database</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="A182" t="str">
-        <v>181</v>
-      </c>
-      <c r="B182" t="str">
-        <v>UT-181</v>
-      </c>
-      <c r="C182" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D182" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E182" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F182" t="str">
-        <v>test_inventory_missing_paths_creates_nothing</v>
-      </c>
-      <c r="G182" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H182" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I182" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J182" t="str">
-        <v>tests/test_preflight.py::test_inventory_missing_paths_creates_nothing</v>
-      </c>
-      <c r="K182" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L182"/>
-      <c r="M182"/>
-      <c r="N182"/>
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>181</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>UT-181</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>test_inventory_missing_paths_creates_nothing</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_inventory_missing_paths_creates_nothing</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="183">
-      <c r="A183" t="str">
-        <v>182</v>
-      </c>
-      <c r="B183" t="str">
-        <v>UT-182</v>
-      </c>
-      <c r="C183" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D183" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E183" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F183" t="str">
-        <v>test_inventory_parses_whitelisted_fields_only</v>
-      </c>
-      <c r="G183" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H183" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I183" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J183" t="str">
-        <v>tests/test_preflight.py::test_inventory_parses_whitelisted_fields_only</v>
-      </c>
-      <c r="K183" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L183"/>
-      <c r="M183"/>
-      <c r="N183"/>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>182</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>UT-182</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>test_inventory_parses_whitelisted_fields_only</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_inventory_parses_whitelisted_fields_only</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="184">
-      <c r="A184" t="str">
-        <v>183</v>
-      </c>
-      <c r="B184" t="str">
-        <v>UT-183</v>
-      </c>
-      <c r="C184" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D184" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E184" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F184" t="str">
-        <v>test_symlink_metadata_does_not_follow_target</v>
-      </c>
-      <c r="G184" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H184" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I184" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J184" t="str">
-        <v>tests/test_preflight.py::test_symlink_metadata_does_not_follow_target</v>
-      </c>
-      <c r="K184" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L184"/>
-      <c r="M184"/>
-      <c r="N184"/>
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>183</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>UT-183</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>test_symlink_metadata_does_not_follow_target</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_symlink_metadata_does_not_follow_target</t>
+        </is>
+      </c>
+      <c r="K184" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="185">
-      <c r="A185" t="str">
-        <v>184</v>
-      </c>
-      <c r="B185" t="str">
-        <v>UT-184</v>
-      </c>
-      <c r="C185" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D185" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E185" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F185" t="str">
-        <v>test_remote_or_credential_urls_are_rejected</v>
-      </c>
-      <c r="G185" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H185" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I185" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J185" t="str">
-        <v>tests/test_preflight.py::test_remote_or_credential_urls_are_rejected</v>
-      </c>
-      <c r="K185" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L185"/>
-      <c r="M185"/>
-      <c r="N185"/>
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>184</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>UT-184</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>test_remote_or_credential_urls_are_rejected</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_remote_or_credential_urls_are_rejected</t>
+        </is>
+      </c>
+      <c r="K185" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="186">
-      <c r="A186" t="str">
-        <v>185</v>
-      </c>
-      <c r="B186" t="str">
-        <v>UT-185</v>
-      </c>
-      <c r="C186" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D186" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E186" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F186" t="str">
-        <v>test_metadata_checks_never_generate</v>
-      </c>
-      <c r="G186" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H186" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I186" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J186" t="str">
-        <v>tests/test_preflight.py::test_metadata_checks_never_generate</v>
-      </c>
-      <c r="K186" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L186"/>
-      <c r="M186"/>
-      <c r="N186"/>
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>185</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>UT-185</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>test_metadata_checks_never_generate</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_metadata_checks_never_generate</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="187">
-      <c r="A187" t="str">
-        <v>186</v>
-      </c>
-      <c r="B187" t="str">
-        <v>UT-186</v>
-      </c>
-      <c r="C187" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D187" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E187" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F187" t="str">
-        <v>test_inference_is_explicit_bounded_local_and_sanitized</v>
-      </c>
-      <c r="G187" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H187" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I187" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J187" t="str">
-        <v>tests/test_preflight.py::test_inference_is_explicit_bounded_local_and_sanitized</v>
-      </c>
-      <c r="K187" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L187"/>
-      <c r="M187"/>
-      <c r="N187"/>
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>186</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>UT-186</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>test_inference_is_explicit_bounded_local_and_sanitized</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_inference_is_explicit_bounded_local_and_sanitized</t>
+        </is>
+      </c>
+      <c r="K187" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="188">
-      <c r="A188" t="str">
-        <v>187</v>
-      </c>
-      <c r="B188" t="str">
-        <v>UT-187</v>
-      </c>
-      <c r="C188" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D188" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E188" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F188" t="str">
-        <v>test_bad_cli_options_fail_without_inventory</v>
-      </c>
-      <c r="G188" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H188" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I188" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J188" t="str">
-        <v>tests/test_preflight.py::test_bad_cli_options_fail_without_inventory</v>
-      </c>
-      <c r="K188" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L188"/>
-      <c r="M188"/>
-      <c r="N188"/>
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>UT-187</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>test_bad_cli_options_fail_without_inventory</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_bad_cli_options_fail_without_inventory</t>
+        </is>
+      </c>
+      <c r="K188" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="189">
-      <c r="A189" t="str">
-        <v>188</v>
-      </c>
-      <c r="B189" t="str">
-        <v>UT-188</v>
-      </c>
-      <c r="C189" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D189" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E189" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F189" t="str">
-        <v>test_command_errors_are_sanitized</v>
-      </c>
-      <c r="G189" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H189" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I189" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J189" t="str">
-        <v>tests/test_preflight.py::test_command_errors_are_sanitized</v>
-      </c>
-      <c r="K189" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L189"/>
-      <c r="M189"/>
-      <c r="N189"/>
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>188</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>UT-188</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>test_command_errors_are_sanitized</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_command_errors_are_sanitized</t>
+        </is>
+      </c>
+      <c r="K189" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="190">
-      <c r="A190" t="str">
-        <v>189</v>
-      </c>
-      <c r="B190" t="str">
-        <v>UT-189</v>
-      </c>
-      <c r="C190" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D190" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E190" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F190" t="str">
-        <v>test_remote_docker_context_is_not_reported_as_local</v>
-      </c>
-      <c r="G190" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H190" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I190" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J190" t="str">
-        <v>tests/test_preflight.py::test_remote_docker_context_is_not_reported_as_local</v>
-      </c>
-      <c r="K190" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L190"/>
-      <c r="M190"/>
-      <c r="N190"/>
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>189</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>UT-189</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>test_remote_docker_context_is_not_reported_as_local</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_remote_docker_context_is_not_reported_as_local</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="191">
-      <c r="A191" t="str">
-        <v>190</v>
-      </c>
-      <c r="B191" t="str">
-        <v>UT-190</v>
-      </c>
-      <c r="C191" t="str">
-        <v>REQ-PREFLIGHT</v>
-      </c>
-      <c r="D191" t="str">
-        <v>로컬 준비 상태 진단</v>
-      </c>
-      <c r="E191" t="str">
-        <v>단위/CLI</v>
-      </c>
-      <c r="F191" t="str">
-        <v>test_docker_host_override_is_not_contacted</v>
-      </c>
-      <c r="G191" t="str">
-        <v>격리 임시 디렉터리·가짜 서비스</v>
-      </c>
-      <c r="H191" t="str">
-        <v>상태·URL·네트워크 조건별 진단</v>
-      </c>
-      <c r="I191" t="str">
-        <v>비밀 미출력·기존 데이터 보존·명시적 추론</v>
-      </c>
-      <c r="J191" t="str">
-        <v>tests/test_preflight.py::test_docker_host_override_is_not_contacted</v>
-      </c>
-      <c r="K191" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L191"/>
-      <c r="M191"/>
-      <c r="N191"/>
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>UT-190</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>REQ-PREFLIGHT</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>로컬 준비 상태 진단</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>단위/CLI</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>test_docker_host_override_is_not_contacted</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>격리 임시 디렉터리·가짜 서비스</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>상태·URL·네트워크 조건별 진단</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>비밀 미출력·기존 데이터 보존·명시적 추론</t>
+        </is>
+      </c>
+      <c r="J191" t="inlineStr">
+        <is>
+          <t>tests/test_preflight.py::test_docker_host_override_is_not_contacted</t>
+        </is>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="192">
-      <c r="A192" t="str">
-        <v>191</v>
-      </c>
-      <c r="B192" t="str">
-        <v>UT-191</v>
-      </c>
-      <c r="C192" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D192" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E192" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F192" t="str">
-        <v>test_judge_feedback_strict_schema</v>
-      </c>
-      <c r="G192" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H192" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I192" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J192" t="str">
-        <v>tests/test_ai_judge.py::test_judge_feedback_strict_schema</v>
-      </c>
-      <c r="K192" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L192"/>
-      <c r="M192"/>
-      <c r="N192"/>
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>191</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>UT-191</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>test_judge_feedback_strict_schema</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J192" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_judge_feedback_strict_schema</t>
+        </is>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="193">
-      <c r="A193" t="str">
-        <v>192</v>
-      </c>
-      <c r="B193" t="str">
-        <v>UT-192</v>
-      </c>
-      <c r="C193" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D193" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E193" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F193" t="str">
-        <v>test_reward_weighting_uncertainty_and_zero_constraints</v>
-      </c>
-      <c r="G193" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H193" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I193" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J193" t="str">
-        <v>tests/test_ai_judge.py::test_reward_weighting_uncertainty_and_zero_constraints</v>
-      </c>
-      <c r="K193" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L193"/>
-      <c r="M193"/>
-      <c r="N193"/>
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>192</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>UT-192</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>test_reward_weighting_uncertainty_and_zero_constraints</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_reward_weighting_uncertainty_and_zero_constraints</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="194">
-      <c r="A194" t="str">
-        <v>193</v>
-      </c>
-      <c r="B194" t="str">
-        <v>UT-193</v>
-      </c>
-      <c r="C194" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D194" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E194" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F194" t="str">
-        <v>test_judge_failures_never_become_zero_rewards</v>
-      </c>
-      <c r="G194" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H194" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I194" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J194" t="str">
-        <v>tests/test_ai_judge.py::test_judge_failures_never_become_zero_rewards</v>
-      </c>
-      <c r="K194" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L194"/>
-      <c r="M194"/>
-      <c r="N194"/>
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>193</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>UT-193</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>test_judge_failures_never_become_zero_rewards</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_judge_failures_never_become_zero_rewards</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="195">
-      <c r="A195" t="str">
-        <v>194</v>
-      </c>
-      <c r="B195" t="str">
-        <v>UT-194</v>
-      </c>
-      <c r="C195" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D195" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E195" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F195" t="str">
-        <v>test_pinning_calibration_and_budget</v>
-      </c>
-      <c r="G195" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H195" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I195" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J195" t="str">
-        <v>tests/test_ai_judge.py::test_pinning_calibration_and_budget</v>
-      </c>
-      <c r="K195" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L195"/>
-      <c r="M195"/>
-      <c r="N195"/>
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>194</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>UT-194</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>test_pinning_calibration_and_budget</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I195" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J195" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_pinning_calibration_and_budget</t>
+        </is>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="196">
-      <c r="A196" t="str">
-        <v>195</v>
-      </c>
-      <c r="B196" t="str">
-        <v>UT-195</v>
-      </c>
-      <c r="C196" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D196" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E196" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F196" t="str">
-        <v>test_judge_local_endpoint_only</v>
-      </c>
-      <c r="G196" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H196" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I196" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J196" t="str">
-        <v>tests/test_ai_judge.py::test_judge_local_endpoint_only</v>
-      </c>
-      <c r="K196" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L196"/>
-      <c r="M196"/>
-      <c r="N196"/>
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>195</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>UT-195</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>test_judge_local_endpoint_only</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I196" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J196" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_judge_local_endpoint_only</t>
+        </is>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="197">
-      <c r="A197" t="str">
-        <v>196</v>
-      </c>
-      <c r="B197" t="str">
-        <v>UT-196</v>
-      </c>
-      <c r="C197" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D197" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E197" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F197" t="str">
-        <v>test_judge_disabled_and_deadline_guards</v>
-      </c>
-      <c r="G197" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H197" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I197" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J197" t="str">
-        <v>tests/test_ai_judge.py::test_judge_disabled_and_deadline_guards</v>
-      </c>
-      <c r="K197" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L197"/>
-      <c r="M197"/>
-      <c r="N197"/>
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>UT-196</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>test_judge_disabled_and_deadline_guards</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I197" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_judge_disabled_and_deadline_guards</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="198">
-      <c r="A198" t="str">
-        <v>197</v>
-      </c>
-      <c r="B198" t="str">
-        <v>UT-197</v>
-      </c>
-      <c r="C198" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D198" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E198" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F198" t="str">
-        <v>test_reward_recorder_preserves_exact_rollouts_and_step</v>
-      </c>
-      <c r="G198" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H198" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I198" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J198" t="str">
-        <v>tests/test_ai_judge.py::test_reward_recorder_preserves_exact_rollouts_and_step</v>
-      </c>
-      <c r="K198" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L198"/>
-      <c r="M198"/>
-      <c r="N198"/>
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>197</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>UT-197</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>test_reward_recorder_preserves_exact_rollouts_and_step</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I198" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J198" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_reward_recorder_preserves_exact_rollouts_and_step</t>
+        </is>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="199">
-      <c r="A199" t="str">
-        <v>198</v>
-      </c>
-      <c r="B199" t="str">
-        <v>UT-198</v>
-      </c>
-      <c r="C199" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D199" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E199" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F199" t="str">
-        <v>test_recorder_failure_does_not_write_fabricated_reward</v>
-      </c>
-      <c r="G199" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H199" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I199" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J199" t="str">
-        <v>tests/test_ai_judge.py::test_recorder_failure_does_not_write_fabricated_reward</v>
-      </c>
-      <c r="K199" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L199"/>
-      <c r="M199"/>
-      <c r="N199"/>
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>198</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>UT-198</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>test_recorder_failure_does_not_write_fabricated_reward</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I199" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>tests/test_ai_judge.py::test_recorder_failure_does_not_write_fabricated_reward</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="200">
-      <c r="A200" t="str">
-        <v>199</v>
-      </c>
-      <c r="B200" t="str">
-        <v>UT-199</v>
-      </c>
-      <c r="C200" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D200" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E200" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F200" t="str">
-        <v>test_rlaif_approval_without_paid_orchestrator</v>
-      </c>
-      <c r="G200" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H200" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I200" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J200" t="str">
-        <v>tests/test_rlaif.py::test_rlaif_approval_without_paid_orchestrator</v>
-      </c>
-      <c r="K200" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L200"/>
-      <c r="M200"/>
-      <c r="N200"/>
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>199</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>UT-199</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr">
+        <is>
+          <t>test_rlaif_approval_without_paid_orchestrator</t>
+        </is>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I200" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_rlaif_approval_without_paid_orchestrator</t>
+        </is>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="201">
-      <c r="A201" t="str">
-        <v>200</v>
-      </c>
-      <c r="B201" t="str">
-        <v>UT-200</v>
-      </c>
-      <c r="C201" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D201" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E201" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F201" t="str">
-        <v>test_rlaif_plan_gates</v>
-      </c>
-      <c r="G201" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H201" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I201" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J201" t="str">
-        <v>tests/test_rlaif.py::test_rlaif_plan_gates</v>
-      </c>
-      <c r="K201" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L201"/>
-      <c r="M201"/>
-      <c r="N201"/>
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>UT-200</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr">
+        <is>
+          <t>test_rlaif_plan_gates</t>
+        </is>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I201" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_rlaif_plan_gates</t>
+        </is>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="202">
-      <c r="A202" t="str">
-        <v>201</v>
-      </c>
-      <c r="B202" t="str">
-        <v>UT-201</v>
-      </c>
-      <c r="C202" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D202" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E202" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F202" t="str">
-        <v>test_disabled_rlaif_does_not_reuse_sft_permission</v>
-      </c>
-      <c r="G202" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H202" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I202" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J202" t="str">
-        <v>tests/test_rlaif.py::test_disabled_rlaif_does_not_reuse_sft_permission</v>
-      </c>
-      <c r="K202" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L202"/>
-      <c r="M202"/>
-      <c r="N202"/>
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>UT-201</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr">
+        <is>
+          <t>test_disabled_rlaif_does_not_reuse_sft_permission</t>
+        </is>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I202" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_disabled_rlaif_does_not_reuse_sft_permission</t>
+        </is>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="203">
-      <c r="A203" t="str">
-        <v>202</v>
-      </c>
-      <c r="B203" t="str">
-        <v>UT-202</v>
-      </c>
-      <c r="C203" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D203" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E203" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F203" t="str">
-        <v>test_failed_calibration_preserves_previous_approval</v>
-      </c>
-      <c r="G203" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H203" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I203" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J203" t="str">
-        <v>tests/test_rlaif.py::test_failed_calibration_preserves_previous_approval</v>
-      </c>
-      <c r="K203" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L203"/>
-      <c r="M203"/>
-      <c r="N203"/>
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>202</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>UT-202</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>test_failed_calibration_preserves_previous_approval</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I203" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J203" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_failed_calibration_preserves_previous_approval</t>
+        </is>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="204">
-      <c r="A204" t="str">
-        <v>203</v>
-      </c>
-      <c r="B204" t="str">
-        <v>UT-203</v>
-      </c>
-      <c r="C204" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D204" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E204" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F204" t="str">
-        <v>test_worker_dispatches_current_policy_training_without_activation</v>
-      </c>
-      <c r="G204" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H204" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I204" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J204" t="str">
-        <v>tests/test_rlaif.py::test_worker_dispatches_current_policy_training_without_activation</v>
-      </c>
-      <c r="K204" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L204"/>
-      <c r="M204"/>
-      <c r="N204"/>
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>203</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>UT-203</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>test_worker_dispatches_current_policy_training_without_activation</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_worker_dispatches_current_policy_training_without_activation</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="205">
-      <c r="A205" t="str">
-        <v>204</v>
-      </c>
-      <c r="B205" t="str">
-        <v>UT-204</v>
-      </c>
-      <c r="C205" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D205" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E205" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F205" t="str">
-        <v>test_worker_rejects_revoked_rlaif_before_training</v>
-      </c>
-      <c r="G205" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H205" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I205" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J205" t="str">
-        <v>tests/test_rlaif.py::test_worker_rejects_revoked_rlaif_before_training</v>
-      </c>
-      <c r="K205" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L205"/>
-      <c r="M205"/>
-      <c r="N205"/>
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>204</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>UT-204</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>test_worker_rejects_revoked_rlaif_before_training</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I205" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J205" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_worker_rejects_revoked_rlaif_before_training</t>
+        </is>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="206">
-      <c r="A206" t="str">
-        <v>205</v>
-      </c>
-      <c r="B206" t="str">
-        <v>UT-205</v>
-      </c>
-      <c r="C206" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D206" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E206" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F206" t="str">
-        <v>test_parent_sft_adapter_is_pinned_and_revalidated</v>
-      </c>
-      <c r="G206" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H206" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I206" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J206" t="str">
-        <v>tests/test_rlaif.py::test_parent_sft_adapter_is_pinned_and_revalidated</v>
-      </c>
-      <c r="K206" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L206"/>
-      <c r="M206"/>
-      <c r="N206"/>
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>205</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>UT-205</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>test_parent_sft_adapter_is_pinned_and_revalidated</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_parent_sft_adapter_is_pinned_and_revalidated</t>
+        </is>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="207">
-      <c r="A207" t="str">
-        <v>206</v>
-      </c>
-      <c r="B207" t="str">
-        <v>UT-206</v>
-      </c>
-      <c r="C207" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D207" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E207" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F207" t="str">
-        <v>test_preview_requires_consent_owner_and_does_not_enqueue</v>
-      </c>
-      <c r="G207" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H207" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I207" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J207" t="str">
-        <v>tests/test_rlaif.py::test_preview_requires_consent_owner_and_does_not_enqueue</v>
-      </c>
-      <c r="K207" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L207"/>
-      <c r="M207"/>
-      <c r="N207"/>
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>206</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>UT-206</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>test_preview_requires_consent_owner_and_does_not_enqueue</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J207" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_preview_requires_consent_owner_and_does_not_enqueue</t>
+        </is>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="208">
-      <c r="A208" t="str">
-        <v>207</v>
-      </c>
-      <c r="B208" t="str">
-        <v>UT-207</v>
-      </c>
-      <c r="C208" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D208" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E208" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F208" t="str">
-        <v>test_candidate_rejects_unqualified_rlaif</v>
-      </c>
-      <c r="G208" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H208" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I208" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J208" t="str">
-        <v>tests/test_rlaif.py::test_candidate_rejects_unqualified_rlaif</v>
-      </c>
-      <c r="K208" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L208"/>
-      <c r="M208"/>
-      <c r="N208"/>
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>207</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>UT-207</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>test_candidate_rejects_unqualified_rlaif</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J208" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_candidate_rejects_unqualified_rlaif</t>
+        </is>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="209">
-      <c r="A209" t="str">
-        <v>208</v>
-      </c>
-      <c r="B209" t="str">
-        <v>UT-208</v>
-      </c>
-      <c r="C209" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D209" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E209" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F209" t="str">
-        <v>test_reward_history_is_owner_bound_and_hash_checked</v>
-      </c>
-      <c r="G209" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H209" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I209" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J209" t="str">
-        <v>tests/test_rlaif.py::test_reward_history_is_owner_bound_and_hash_checked</v>
-      </c>
-      <c r="K209" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L209"/>
-      <c r="M209"/>
-      <c r="N209"/>
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>208</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>UT-208</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>test_reward_history_is_owner_bound_and_hash_checked</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I209" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_reward_history_is_owner_bound_and_hash_checked</t>
+        </is>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="210">
-      <c r="A210" t="str">
-        <v>209</v>
-      </c>
-      <c r="B210" t="str">
-        <v>UT-209</v>
-      </c>
-      <c r="C210" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D210" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E210" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F210" t="str">
-        <v>test_grpo_generation_settings_and_long_prompt_rejection</v>
-      </c>
-      <c r="G210" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H210" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I210" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J210" t="str">
-        <v>tests/test_rlaif.py::test_grpo_generation_settings_and_long_prompt_rejection</v>
-      </c>
-      <c r="K210" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L210"/>
-      <c r="M210"/>
-      <c r="N210"/>
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>209</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>UT-209</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>test_grpo_generation_settings_and_long_prompt_rejection</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I210" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J210" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_grpo_generation_settings_and_long_prompt_rejection</t>
+        </is>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
     <row r="211">
-      <c r="A211" t="str">
-        <v>210</v>
-      </c>
-      <c r="B211" t="str">
-        <v>UT-210</v>
-      </c>
-      <c r="C211" t="str">
-        <v>REQ-RLAIF</v>
-      </c>
-      <c r="D211" t="str">
-        <v>AI 피드백 강화학습</v>
-      </c>
-      <c r="E211" t="str">
-        <v>단위/API</v>
-      </c>
-      <c r="F211" t="str">
-        <v>test_resource_retry_preserves_partial_attempt</v>
-      </c>
-      <c r="G211" t="str">
-        <v>합성 평가·격리 데이터</v>
-      </c>
-      <c r="H211" t="str">
-        <v>정책·보상·승인·작업·후보 조건 검사</v>
-      </c>
-      <c r="I211" t="str">
-        <v>무권한 실행 차단·기록 보존·보상 무결성</v>
-      </c>
-      <c r="J211" t="str">
-        <v>tests/test_rlaif.py::test_resource_retry_preserves_partial_attempt</v>
-      </c>
-      <c r="K211" t="str">
-        <v>미실행</v>
-      </c>
-      <c r="L211"/>
-      <c r="M211"/>
-      <c r="N211"/>
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>UT-210</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>REQ-RLAIF</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>AI 피드백 강화학습</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>test_resource_retry_preserves_partial_attempt</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>합성 평가·격리 데이터</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>정책·보상·승인·작업·후보 조건 검사</t>
+        </is>
+      </c>
+      <c r="I211" t="inlineStr">
+        <is>
+          <t>무권한 실행 차단·기록 보존·보상 무결성</t>
+        </is>
+      </c>
+      <c r="J211" t="inlineStr">
+        <is>
+          <t>tests/test_rlaif.py::test_resource_retry_preserves_partial_attempt</t>
+        </is>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>211</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>UT-211</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>test_six_definitions_resolve_existing_models_without_execution</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I212" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_six_definitions_resolve_existing_models_without_execution</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>212</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>UT-212</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>test_schema_rejects_unsupported_or_unsafe_settings</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I213" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_schema_rejects_unsupported_or_unsafe_settings</t>
+        </is>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>213</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>UT-213</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>test_explicit_configuration_is_not_ignored_and_has_no_raw_error_leak</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I214" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_explicit_configuration_is_not_ignored_and_has_no_raw_error_leak</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>214</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>UT-214</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>test_path_escape_rejected</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I215" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_path_escape_rejected</t>
+        </is>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>215</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>UT-215</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>test_symlink_large_file_and_duplicate_keys_rejected</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I216" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J216" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_symlink_large_file_and_duplicate_keys_rejected</t>
+        </is>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>216</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>UT-216</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>test_invalid_config_rejected_before_database_creation</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_invalid_config_rejected_before_database_creation</t>
+        </is>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>217</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>UT-217</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>test_api_auth_owner_no_store_and_no_mutation</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_api_auth_owner_no_store_and_no_mutation</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>218</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>UT-218</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>test_api_requires_authentication</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_api_requires_authentication</t>
+        </is>
+      </c>
+      <c r="K219" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>219</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>UT-219</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>test_chat_keeps_one_provider_call_without_registry_dispatch</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I220" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J220" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_chat_keeps_one_provider_call_without_registry_dispatch</t>
+        </is>
+      </c>
+      <c r="K220" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>UT-220</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>test_public_mode_cannot_list_definitions</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I221" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J221" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_public_mode_cannot_list_definitions</t>
+        </is>
+      </c>
+      <c r="K221" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>221</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>UT-221</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>test_parallelism_limit_does_not_accept_boolean_or_float</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_parallelism_limit_does_not_accept_boolean_or_float</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>UT-222</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>test_nested_invalid_json_has_safe_error</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I223" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J223" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_nested_invalid_json_has_safe_error</t>
+        </is>
+      </c>
+      <c r="K223" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>223</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>UT-223</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>test_config_directory_symlink_rejected</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_config_directory_symlink_rejected</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>224</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>UT-224</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>역할 구성·권한 경계</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>test_configured_restrictions_and_existing_coding_model_are_reflected</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>tests/test_agent_registry.py::test_configured_restrictions_and_existing_coding_model_are_reflected</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>225</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>UT-225</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>REQ-BASELINE</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>읽기 전용 기준선</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>test_manifest_is_hashes_only_and_distinguishes_runtime_and_performance</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I226" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>tests/test_baseline_manifest.py::test_manifest_is_hashes_only_and_distinguishes_runtime_and_performance</t>
+        </is>
+      </c>
+      <c r="K226" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>226</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>UT-226</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>REQ-BASELINE</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>읽기 전용 기준선</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>test_source_change_changes_identity</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I227" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t>tests/test_baseline_manifest.py::test_source_change_changes_identity</t>
+        </is>
+      </c>
+      <c r="K227" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>227</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>UT-227</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>REQ-BASELINE</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>읽기 전용 기준선</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>test_source_symlink_rejected</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I228" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>tests/test_baseline_manifest.py::test_source_symlink_rejected</t>
+        </is>
+      </c>
+      <c r="K228" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>228</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>UT-228</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>REQ-BASELINE</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>읽기 전용 기준선</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>test_cli_never_overwrites_existing_report</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I229" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t>tests/test_baseline_manifest.py::test_cli_never_overwrites_existing_report</t>
+        </is>
+      </c>
+      <c r="K229" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N211"/>
+  <autoFilter ref="A1:N229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12009,7 +13600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12332,6 +13923,40 @@
       <c r="C19" t="inlineStr">
         <is>
           <t>자동 검증; 실제 GPU 생성·배포는 별도</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>REQ-AGENT-CONFIG</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>여섯 역할 정의/설정 검증/권한 확대 차단/로컬 소유자 조회/기존 대화 유지</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>REQ-BASELINE</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>소스·설정 해시/Git 식별/원문·비밀 제외/기존 보고서 덮어쓰기 방지</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add approved coding task contracts and isolated workspaces
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$242</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>228개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>241개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N229"/>
+  <dimension ref="A1:N242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13588,8 +13588,749 @@
         </is>
       </c>
     </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>229</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>UT-229</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>test_real_worktree_patch_and_source_preservation</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_real_worktree_patch_and_source_preservation</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>UT-230</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>test_forbidden_paths_cannot_be_approved</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H231" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I231" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_forbidden_paths_cannot_be_approved</t>
+        </is>
+      </c>
+      <c r="K231" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>231</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>UT-231</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>test_contracts_reject_coercion_unknown_fields_and_mutation</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H232" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I232" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_contracts_reject_coercion_unknown_fields_and_mutation</t>
+        </is>
+      </c>
+      <c r="K232" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>232</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>UT-232</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>test_approval_binds_owner_project_commit_scope_budget_and_content</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H233" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I233" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_approval_binds_owner_project_commit_scope_budget_and_content</t>
+        </is>
+      </c>
+      <c r="K233" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>233</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>UT-233</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>test_invalid_batches_fail_before_any_write</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H234" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I234" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_invalid_batches_fail_before_any_write</t>
+        </is>
+      </c>
+      <c r="K234" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>234</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>UT-234</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>test_workspace_tampering_is_rejected</t>
+        </is>
+      </c>
+      <c r="G235" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H235" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I235" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J235" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_workspace_tampering_is_rejected</t>
+        </is>
+      </c>
+      <c r="K235" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>235</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>UT-235</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>test_unsupported_repository_rejected_without_workspace</t>
+        </is>
+      </c>
+      <c r="G236" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H236" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I236" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J236" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_unsupported_repository_rejected_without_workspace</t>
+        </is>
+      </c>
+      <c r="K236" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>236</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>UT-236</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>test_checkout_hooks_filters_and_inherited_git_config_never_execute</t>
+        </is>
+      </c>
+      <c r="G237" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H237" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I237" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J237" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_checkout_hooks_filters_and_inherited_git_config_never_execute</t>
+        </is>
+      </c>
+      <c r="K237" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>237</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>UT-237</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>test_deadline_existing_paths_and_private_root</t>
+        </is>
+      </c>
+      <c r="G238" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H238" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I238" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J238" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_deadline_existing_paths_and_private_root</t>
+        </is>
+      </c>
+      <c r="K238" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>238</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>UT-238</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>test_no_final_newline_artifact_is_applyable</t>
+        </is>
+      </c>
+      <c r="G239" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H239" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I239" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J239" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_no_final_newline_artifact_is_applyable</t>
+        </is>
+      </c>
+      <c r="K239" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>239</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>UT-239</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>test_git_errors_do_not_expose_stderr_or_contents</t>
+        </is>
+      </c>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H240" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I240" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_git_errors_do_not_expose_stderr_or_contents</t>
+        </is>
+      </c>
+      <c r="K240" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>240</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>UT-240</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>test_partial_write_failure_is_blocked_and_source_untouched</t>
+        </is>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H241" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I241" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_partial_write_failure_is_blocked_and_source_untouched</t>
+        </is>
+      </c>
+      <c r="K241" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>241</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>UT-241</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>코딩 작업·격리 파일 변경</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>test_concurrent_application_is_rejected</t>
+        </is>
+      </c>
+      <c r="G242" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H242" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J242" t="inlineStr">
+        <is>
+          <t>tests/test_coding_workspace.py::test_concurrent_application_is_rejected</t>
+        </is>
+      </c>
+      <c r="K242" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N229"/>
+  <autoFilter ref="A1:N242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13600,7 +14341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13955,6 +14696,23 @@
         </is>
       </c>
       <c r="C21" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>REQ-CODING-WORKSPACE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>작업·변경 승인 해시/격리 worktree/원본 보존/경로·수정량 제한/실행 금지/diff</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: add opt-in metadata-only coding strategy recorder
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$258</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>241개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>257개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N242"/>
+  <dimension ref="A1:N258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14329,8 +14329,920 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>UT-242</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>test_safe_defaults_and_hidden_evaluation_do_not_touch_sink</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_safe_defaults_and_hidden_evaluation_do_not_touch_sink</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>UT-243</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>test_strict_schema_rejects_raw_or_unverified_payload_without_leak</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_strict_schema_rejects_raw_or_unverified_payload_without_leak</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>UT-244</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>test_adapter_stores_only_selected_fields_and_never_claims_test_success</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_adapter_stores_only_selected_fields_and_never_claims_test_success</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>UT-245</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>test_phase_outcomes_preserve_unknown_and_failure</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_phase_outcomes_preserve_unknown_and_failure</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>UT-246</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>test_state_invariants_cannot_be_forged</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_state_invariants_cannot_be_forged</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>UT-247</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>test_idempotency_conflicts_capacity_and_sequence_arrival_order</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_idempotency_conflicts_capacity_and_sequence_arrival_order</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>UT-248</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>test_workspace_retries_keep_original_id_timestamp_and_content</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_workspace_retries_keep_original_id_timestamp_and_content</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>UT-249</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>test_cross_scope_events_rejected_and_private_snapshot_gated</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_cross_scope_events_rejected_and_private_snapshot_gated</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>UT-250</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>test_consent_snapshot_mismatch_unknown_state_and_attempt_limit</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_consent_snapshot_mismatch_unknown_state_and_attempt_limit</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>UT-251</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>test_sink_failures_and_busy_buffer_are_bounded_safe_receipts</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_sink_failures_and_busy_buffer_are_bounded_safe_receipts</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>UT-252</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>test_model_construct_bypass_and_immutable_snapshots</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_model_construct_bypass_and_immutable_snapshots</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>UT-253</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>test_memory_limits_are_strict_and_bounded</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_memory_limits_are_strict_and_bounded</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>UT-254</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>test_policy_flags_are_strict_and_unbounded_custom_sinks_rejected</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_policy_flags_are_strict_and_unbounded_custom_sinks_rejected</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>UT-255</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>test_concurrent_duplicates_do_not_inflate_memory</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_concurrent_duplicates_do_not_inflate_memory</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>UT-256</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>test_recording_has_no_filesystem_process_network_or_database_side_effects</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_recording_has_no_filesystem_process_network_or_database_side_effects</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>UT-257</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>최소 전략 경험·메모리 기록</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>test_real_workspace_off_on_and_recorder_failure_preserve_patch_and_approval</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_real_workspace_off_on_and_recorder_failure_preserve_patch_and_approval</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N242"/>
+  <autoFilter ref="A1:N258"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14341,7 +15253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14713,6 +15625,23 @@
         </is>
       </c>
       <c r="C22" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>민감 원문 차단/동의·범위/상태/멱등·용량·장애/기록 off-on 코드·승인 불변</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: implement checkpointed local coding agent runtime
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$273</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>241개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>272개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N242"/>
+  <dimension ref="A1:N273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14329,8 +14329,1775 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>UT-242</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>test_safe_defaults_and_hidden_evaluation_do_not_touch_sink</t>
+        </is>
+      </c>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H243" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_safe_defaults_and_hidden_evaluation_do_not_touch_sink</t>
+        </is>
+      </c>
+      <c r="K243" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>243</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>UT-243</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>test_strict_schema_rejects_raw_or_unverified_payload_without_leak</t>
+        </is>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I244" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J244" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_strict_schema_rejects_raw_or_unverified_payload_without_leak</t>
+        </is>
+      </c>
+      <c r="K244" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>244</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>UT-244</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>test_adapter_stores_only_selected_fields_and_never_claims_test_success</t>
+        </is>
+      </c>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H245" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_adapter_stores_only_selected_fields_and_never_claims_test_success</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>245</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>UT-245</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>test_phase_outcomes_preserve_unknown_and_failure</t>
+        </is>
+      </c>
+      <c r="G246" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H246" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I246" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J246" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_phase_outcomes_preserve_unknown_and_failure</t>
+        </is>
+      </c>
+      <c r="K246" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>246</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>UT-246</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>test_state_invariants_cannot_be_forged</t>
+        </is>
+      </c>
+      <c r="G247" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H247" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I247" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J247" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_state_invariants_cannot_be_forged</t>
+        </is>
+      </c>
+      <c r="K247" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>247</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>UT-247</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>test_idempotency_conflicts_capacity_and_sequence_arrival_order</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I248" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J248" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_idempotency_conflicts_capacity_and_sequence_arrival_order</t>
+        </is>
+      </c>
+      <c r="K248" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>248</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>UT-248</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>test_workspace_retries_keep_original_id_timestamp_and_content</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J249" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_workspace_retries_keep_original_id_timestamp_and_content</t>
+        </is>
+      </c>
+      <c r="K249" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>249</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>UT-249</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>test_cross_scope_events_rejected_and_private_snapshot_gated</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_cross_scope_events_rejected_and_private_snapshot_gated</t>
+        </is>
+      </c>
+      <c r="K250" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>UT-250</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>test_consent_snapshot_mismatch_unknown_state_and_attempt_limit</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I251" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_consent_snapshot_mismatch_unknown_state_and_attempt_limit</t>
+        </is>
+      </c>
+      <c r="K251" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>251</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>UT-251</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>test_sink_failures_and_busy_buffer_are_bounded_safe_receipts</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I252" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J252" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_sink_failures_and_busy_buffer_are_bounded_safe_receipts</t>
+        </is>
+      </c>
+      <c r="K252" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>252</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>UT-252</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>test_model_construct_bypass_and_immutable_snapshots</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I253" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J253" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_model_construct_bypass_and_immutable_snapshots</t>
+        </is>
+      </c>
+      <c r="K253" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>253</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>UT-253</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>test_memory_limits_are_strict_and_bounded</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I254" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_memory_limits_are_strict_and_bounded</t>
+        </is>
+      </c>
+      <c r="K254" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>254</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>UT-254</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>test_policy_flags_are_strict_and_unbounded_custom_sinks_rejected</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I255" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J255" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_policy_flags_are_strict_and_unbounded_custom_sinks_rejected</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>255</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>UT-255</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>test_concurrent_duplicates_do_not_inflate_memory</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I256" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J256" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_concurrent_duplicates_do_not_inflate_memory</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>256</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>UT-256</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>test_recording_has_no_filesystem_process_network_or_database_side_effects</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J257" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_recording_has_no_filesystem_process_network_or_database_side_effects</t>
+        </is>
+      </c>
+      <c r="K257" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>257</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>UT-257</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>최소 전략 경험 기록</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>test_real_workspace_off_on_and_recorder_failure_preserve_patch_and_approval</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I258" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J258" t="inlineStr">
+        <is>
+          <t>tests/test_strategy_events.py::test_real_workspace_off_on_and_recorder_failure_preserve_patch_and_approval</t>
+        </is>
+      </c>
+      <c r="K258" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>258</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>UT-258</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>test_real_git_iterative_fix_test_repair_checkpoint_and_binary_preservation</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I259" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J259" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_real_git_iterative_fix_test_repair_checkpoint_and_binary_preservation</t>
+        </is>
+      </c>
+      <c r="K259" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>259</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>UT-259</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>test_pause_restart_resume_keeps_code_counters_and_budget</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I260" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J260" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_pause_restart_resume_keeps_code_counters_and_budget</t>
+        </is>
+      </c>
+      <c r="K260" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>UT-260</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>test_repeated_error_stops_even_when_model_offers_more_patches</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I261" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J261" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_repeated_error_stops_even_when_model_offers_more_patches</t>
+        </is>
+      </c>
+      <c r="K261" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>261</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>UT-261</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>test_budget_survives_resume_and_no_extra_call_occurs</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J262" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_budget_survives_resume_and_no_extra_call_occurs</t>
+        </is>
+      </c>
+      <c r="K262" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>262</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>UT-262</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>test_crash_unknown_step_requires_ack_and_reserves_resources</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J263" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_crash_unknown_step_requires_ack_and_reserves_resources</t>
+        </is>
+      </c>
+      <c r="K263" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>263</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>UT-263</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>test_pause_cancel_controls_and_cross_worker_lock</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J264" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_pause_cancel_controls_and_cross_worker_lock</t>
+        </is>
+      </c>
+      <c r="K264" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>264</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>UT-264</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>test_corrupt_checkpoint_owner_and_symlink_are_rejected</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J265" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_corrupt_checkpoint_owner_and_symlink_are_rejected</t>
+        </is>
+      </c>
+      <c r="K265" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>265</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>UT-265</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>test_patch_scope_tests_and_runtime_configuration_cannot_be_bypassed</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_patch_scope_tests_and_runtime_configuration_cannot_be_bypassed</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>266</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>UT-266</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>test_no_false_finish_malformed_actions_and_stale_tests</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_no_false_finish_malformed_actions_and_stale_tests</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>267</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>UT-267</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>test_busy_gpu_does_not_spend_call_reservation_and_cloud_endpoint_is_rejected</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_busy_gpu_does_not_spend_call_reservation_and_cloud_endpoint_is_rejected</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>268</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>UT-268</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>test_recorder_failure_does_not_change_coding_result</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_recorder_failure_does_not_change_coding_result</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>269</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>UT-269</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>test_coding_api_uses_existing_auth_csrf_and_owner_boundaries</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_coding_api_uses_existing_auth_csrf_and_owner_boundaries</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>270</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>UT-270</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>test_repository_runner_limits_evidence_and_cleanup_guard</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_repository_runner_limits_evidence_and_cleanup_guard</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>271</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>UT-271</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>test_checkpoint_write_failure_preserves_previous_revision</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I272" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_checkpoint_write_failure_preserves_previous_revision</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>272</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>UT-272</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>test_gpu_lock_serializes_calls_and_unknown_timeout_blocks_next_inference</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I273" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_gpu_lock_serializes_calls_and_unknown_timeout_blocks_next_inference</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N242"/>
+  <autoFilter ref="A1:N273"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14341,7 +16108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14713,6 +16480,40 @@
         </is>
       </c>
       <c r="C22" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>REQ-STRATEGY-RECORDER</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>최소 메타데이터/범위/장애/비밀 미저장</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>탐색/반복 수정/격리 명령/오류 복구/체크포인트/중단·재개/예산·승인</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
fix: support bounded source reads and exact incremental edits
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$274</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>272개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>273개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N273"/>
+  <dimension ref="A1:N274"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16096,8 +16096,65 @@
         </is>
       </c>
     </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>273</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>UT-273</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>test_exact_replacement_and_bounded_valid_model_context</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I274" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_exact_replacement_and_bounded_valid_model_context</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N273"/>
+  <autoFilter ref="A1:N274"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: constrain coding actions with Ollama JSON schema
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$274</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$275</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>273개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>274개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N274"/>
+  <dimension ref="A1:N275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16153,8 +16153,65 @@
         </is>
       </c>
     </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>274</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>UT-274</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>REQ-CODING-RUNTIME</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>코딩 실행·복구·체크포인트</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>test_local_model_requests_action_schema_instead_of_unconstrained_json</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>tests/test_coding_runtime.py::test_local_model_requests_action_schema_instead_of_unconstrained_json</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N274"/>
+  <autoFilter ref="A1:N275"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
test(coding): register stability scenarios in the Excel QA plan
Import shared fixtures without assuming tests is a package (CI collection error).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$275</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$297</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>274개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>296개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N275"/>
+  <dimension ref="A1:N297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16210,8 +16210,1262 @@
         </is>
       </c>
     </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>275</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>UT-275</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>test_json_escapes_decode_to_real_newlines_and_double_escapes_are_repaired</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I276" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_json_escapes_decode_to_real_newlines_and_double_escapes_are_repaired</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>276</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>UT-276</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>test_crlf_and_missing_final_newline_are_matched_consistently</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I277" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_crlf_and_missing_final_newline_are_matched_consistently</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>277</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>UT-277</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>test_ambiguous_or_missing_text_is_never_patched</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I278" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_ambiguous_or_missing_text_is_never_patched</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>278</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>UT-278</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>test_several_edits_to_one_file_merge_in_order_and_partial_failure_changes_nothing</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I279" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_several_edits_to_one_file_merge_in_order_and_partial_failure_changes_nothing</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>279</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>UT-279</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>test_two_changes_to_same_file_complete_end_to_end</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I280" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_two_changes_to_same_file_complete_end_to_end</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>280</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>UT-280</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>test_patch_mismatch_is_recoverable_and_checkpoint_stays_consistent</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_patch_mismatch_is_recoverable_and_checkpoint_stays_consistent</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>281</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>UT-281</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>test_identical_rejected_patch_stops_instead_of_looping</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_identical_rejected_patch_stops_instead_of_looping</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>282</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>UT-282</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>test_scope_violation_stays_fatal_even_with_recovery</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_scope_violation_stays_fatal_even_with_recovery</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>283</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>UT-283</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>test_finish_without_passing_test_is_rejected_and_never_completes</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_finish_without_passing_test_is_rejected_and_never_completes</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>284</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>UT-284</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>test_response_errors_are_classified</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_response_errors_are_classified</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>285</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>UT-285</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>test_action_json_is_extracted_without_relaxing_the_schema</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_action_json_is_extracted_without_relaxing_the_schema</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>286</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>UT-286</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>test_empty_replies_are_recorded_and_bounded</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_empty_replies_are_recorded_and_bounded</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>287</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>UT-287</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>test_thinking_flag_is_explicit_per_task_and_usage_is_reported</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_thinking_flag_is_explicit_per_task_and_usage_is_reported</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>288</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>UT-288</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>test_keep_alive_is_zero_under_gpu_admission_policy</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_keep_alive_is_zero_under_gpu_admission_policy</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>289</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>UT-289</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>test_release_only_touches_a_resident_model</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_release_only_touches_a_resident_model</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>290</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>UT-290</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>test_measured_usage_replaces_reservation_and_unmeasured_keeps_it</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_measured_usage_replaces_reservation_and_unmeasured_keeps_it</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>291</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>UT-291</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>test_unmeasured_reply_is_charged_the_full_reservation</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_unmeasured_reply_is_charged_the_full_reservation</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>292</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>UT-292</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>test_memory_prevents_reread_and_stops_identical_loops</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_memory_prevents_reread_and_stops_identical_loops</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>293</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>UT-293</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>test_no_progress_alternation_is_bounded</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_no_progress_alternation_is_bounded</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>294</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>UT-294</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>test_memory_survives_pause_resume_and_old_checkpoints_load</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J295" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_memory_survives_pause_resume_and_old_checkpoints_load</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>295</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>UT-295</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>test_model_context_is_bounded_and_test_log_is_digested</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_model_context_is_bounded_and_test_log_is_digested</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>296</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>UT-296</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>코딩 모델 연동·패치 복구·토큰 계측</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>test_new_task_options_validate_and_api_defaults_stay_compatible</t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>tests/test_coding_stability.py::test_new_task_options_validate_and_api_defaults_stay_compatible</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N275"/>
+  <autoFilter ref="A1:N297"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16222,7 +17476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16628,6 +17882,23 @@
         </is>
       </c>
       <c r="C24" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>REQ-CODING-STABILITY</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>thinking 제어/응답 오류 분류/작업 메모리·반복 중단/패치 정규화·복구/실측 토큰 정산/keep_alive</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat(coding): bound context and automate approved revision tests
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$297</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$324</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>296개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>323개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N297"/>
+  <dimension ref="A1:N324"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17464,8 +17464,1547 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>297</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>UT-297</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>test_context_enforces_character_and_utf8_budgets_without_altering_goal</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_context_enforces_character_and_utf8_budgets_without_altering_goal</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>298</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>UT-298</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>test_core_context_overflow_stops_before_inference_or_reservation</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_core_context_overflow_stops_before_inference_or_reservation</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>UT-299</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>test_source_windows_are_verbatim_and_budgeted_including_system_and_output</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_source_windows_are_verbatim_and_budgeted_including_system_and_output</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>UT-300</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>test_context_does_not_silently_truncate_irreducible_task</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_context_does_not_silently_truncate_irreducible_task</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>UT-301</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>test_noop_patch_is_recoverable_and_later_real_fix_completes</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_noop_patch_is_recoverable_and_later_real_fix_completes</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>UT-302</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>test_normalization_preserves_literal_escapes_inside_quoted_source</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_normalization_preserves_literal_escapes_inside_quoted_source</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>UT-303</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>test_patch_mismatch_lists_attempts_but_never_changes_input</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_patch_mismatch_lists_attempts_but_never_changes_input</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>UT-304</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>test_measured_settlement_is_idempotent_and_missing_usage_stays_reserved</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_measured_settlement_is_idempotent_and_missing_usage_stays_reserved</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>UT-305</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>test_timeout_persists_unknown_usage_and_does_not_expose_private_text</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_timeout_persists_unknown_usage_and_does_not_expose_private_text</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>306</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>UT-306</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>test_failed_post_call_checkpoint_keeps_disk_reservation_and_typed_error</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_failed_post_call_checkpoint_keeps_disk_reservation_and_typed_error</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>307</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>UT-307</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>test_repeated_plan_after_real_new_revision_is_not_identical</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_repeated_plan_after_real_new_revision_is_not_identical</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>UT-308</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>test_reply_reports_duration_and_thinking_characters_without_invented_token_count</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_reply_reports_duration_and_thinking_characters_without_invented_token_count</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>UT-309</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>test_benchmark_metrics_separate_success_latency_and_unknown_tokens</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_benchmark_metrics_separate_success_latency_and_unknown_tokens</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>UT-310</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>test_grader_rejects_self_report_without_current_revision_or_protected_files</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_grader_rejects_self_report_without_current_revision_or_protected_files</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>311</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>UT-311</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>test_host_evaluation_rejects_all_skipped_tests</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_host_evaluation_rejects_all_skipped_tests</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>312</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>UT-312</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>test_proven_no_inference_refunds_reservation_and_slot</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_proven_no_inference_refunds_reservation_and_slot</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>UT-313</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>test_deadline_before_send_does_not_charge_unmade_call</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_deadline_before_send_does_not_charge_unmade_call</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>314</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>UT-314</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>test_automatic_tests_complete_with_three_calls_and_real_unittest_evidence</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_automatic_tests_complete_with_three_calls_and_real_unittest_evidence</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>315</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>UT-315</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>test_automatic_test_saves_model_slot_relative_to_same_legacy_budget</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_automatic_test_saves_model_slot_relative_to_same_legacy_budget</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>UT-316</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>test_automatic_test_respects_pause_resume_and_keeps_original_source</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_automatic_test_respects_pause_resume_and_keeps_original_source</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>317</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>UT-317</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>test_automatic_test_cannot_bypass_step_budget</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_automatic_test_cannot_bypass_step_budget</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>UT-318</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>test_interrupted_automatic_test_keeps_pending_and_requires_acknowledgement</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_interrupted_automatic_test_keeps_pending_and_requires_acknowledgement</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>319</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>UT-319</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>test_repeated_tests_on_same_revision_reuse_evidence_without_rerunning</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_repeated_tests_on_same_revision_reuse_evidence_without_rerunning</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>UT-320</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>test_old_approval_does_not_gain_automatic_execution_and_new_tasks_opt_in_by_default</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_old_approval_does_not_gain_automatic_execution_and_new_tasks_opt_in_by_default</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>UT-321</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>test_context_retains_plan_status_without_duplicating_plan_or_source</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_context_retains_plan_status_without_duplicating_plan_or_source</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>UT-322</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>test_suppressed_permission_failure_still_has_safe_structured_code</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_suppressed_permission_failure_still_has_safe_structured_code</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>UT-323</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>REQ-CODING-EVAL</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>컨텍스트·복구·평가 예산 경계</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>test_cached_test_evidence_is_invalidated_by_new_revision</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>tests/test_coding_evaluation.py::test_cached_test_evidence_is_invalidated_by_new_revision</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N297"/>
+  <autoFilter ref="A1:N324"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: add immutable common task contracts and Coding adapters
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$297</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$313</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>296개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>312개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N297"/>
+  <dimension ref="A1:N313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17464,8 +17464,920 @@
         </is>
       </c>
     </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>297</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>UT-297</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>test_invalid_contracts_fail_closed</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_invalid_contracts_fail_closed</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>298</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>UT-298</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>test_personal_scope_is_explicit_and_never_a_wildcard</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_personal_scope_is_explicit_and_never_a_wildcard</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>299</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>UT-299</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>test_resources_require_exact_versions_and_scopes</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_resources_require_exact_versions_and_scopes</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>UT-300</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>test_common_conversion_cannot_bypass_original_coding_paths</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_common_conversion_cannot_bypass_original_coding_paths</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>301</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>UT-301</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>test_resource_identity_cannot_rebind_to_multiple_versions</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_resource_identity_cannot_rebind_to_multiple_versions</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>UT-302</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>test_common_budget_preserves_coding_limits</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_common_budget_preserves_coding_limits</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>303</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>UT-303</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>test_high_risk_requires_human_review_and_models_are_deeply_immutable</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_high_risk_requires_human_review_and_models_are_deeply_immutable</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>304</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>UT-304</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>test_digest_binds_every_immutable_decision</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_digest_binds_every_immutable_decision</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>305</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>UT-305</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>test_digest_is_stable_across_json_order_and_state_updates</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_digest_is_stable_across_json_order_and_state_updates</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>306</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>UT-306</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>test_execution_observations_validate_without_changing_spec</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_execution_observations_validate_without_changing_spec</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>307</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>UT-307</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>test_digest_and_adapter_revalidate_unchecked_model_copies</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_digest_and_adapter_revalidate_unchecked_model_copies</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>308</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>UT-308</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>test_coding_roundtrip_and_legacy_digest_compatibility</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_coding_roundtrip_and_legacy_digest_compatibility</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>309</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>UT-309</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>test_contract_reference_and_success_observation_never_grant_permission</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_contract_reference_and_success_observation_never_grant_permission</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>310</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>UT-310</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>test_runtime_test_files_remain_read_only</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_runtime_test_files_remain_read_only</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>311</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>UT-311</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>test_contract_operations_have_no_io_or_environment_side_effects</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I312" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_contract_operations_have_no_io_or_environment_side_effects</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>312</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>UT-312</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약·Coding 호환</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>단위/계약</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>test_legacy_digest_is_independent_of_new_contract_metadata</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>순수 계약·합성 입력·Mock 권한</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>불변 명세/상태 분리·digest·기존 제한과 호환 검증</t>
+        </is>
+      </c>
+      <c r="I313" t="inlineStr">
+        <is>
+          <t>권한 부여/외부 실행 없음·기존 digest/경로/예산 보존</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>tests/test_task_contracts.py::test_legacy_digest_is_independent_of_new_contract_metadata</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N297"/>
+  <autoFilter ref="A1:N313"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17476,7 +18388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17901,6 +18813,23 @@
       <c r="C25" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>REQ-TASK-CONTRACT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>P1-01 공통 계약/불변 digest/상태 분리/Coding 왕복 호환/권한 비부여</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>자동 검증; 모델·운영 실행 없음</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add project scope metadata and safe migration staging foundation
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$313</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$340</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>312개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>339개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N313"/>
+  <dimension ref="A1:N340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18376,8 +18376,1547 @@
         </is>
       </c>
     </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>313</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>UT-313</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>test_default_private_personal_scope_and_same_name_users</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I314" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_default_private_personal_scope_and_same_name_users</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>314</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>UT-314</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>test_explicit_exact_read_grant_revoke_and_generation</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I315" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_explicit_exact_read_grant_revoke_and_generation</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>315</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>UT-315</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>test_version_change_never_inherits_old_share</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_version_change_never_inherits_old_share</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>316</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>UT-316</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>test_revoked_ancestor_blocks_derived_chain_without_deleting_records</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_revoked_ancestor_blocks_derived_chain_without_deleting_records</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>317</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>UT-317</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>test_cycles_and_cross_user_provenance_are_rejected_by_database</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_cycles_and_cross_user_provenance_are_rejected_by_database</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>318</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>UT-318</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>test_raw_database_cannot_bypass_owner_or_read_version_boundaries</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_raw_database_cannot_bypass_owner_or_read_version_boundaries</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>319</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>UT-319</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>test_scope_history_cannot_be_erased_or_revoked_grants_revived</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_scope_history_cannot_be_erased_or_revoked_grants_revived</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>UT-320</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>test_changed_memory_same_revision_and_inactive_sources_fail_closed</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_changed_memory_same_revision_and_inactive_sources_fail_closed</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>321</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>UT-321</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>test_explicit_alias_mapping_and_p101_resource_reference_compatibility</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_explicit_alias_mapping_and_p101_resource_reference_compatibility</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>322</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>UT-322</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>test_scope_moves_and_archived_target_invalidate_eligibility</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_scope_moves_and_archived_target_invalidate_eligibility</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>UT-323</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>test_memory_revision_carries_revoked_provenance_without_reenabling_it</t>
+        </is>
+      </c>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_memory_revision_carries_revoked_provenance_without_reenabling_it</t>
+        </is>
+      </c>
+      <c r="K324" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>324</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>UT-324</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>test_missing_provenance_on_raw_new_version_never_restores_eligibility</t>
+        </is>
+      </c>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_missing_provenance_on_raw_new_version_never_restores_eligibility</t>
+        </is>
+      </c>
+      <c r="K325" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>UT-325</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>test_archived_origin_blocks_its_shared_versions</t>
+        </is>
+      </c>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_archived_origin_blocks_its_shared_versions</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>326</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>UT-326</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>test_deep_provenance_is_bounded_and_denied_without_recursion_failure</t>
+        </is>
+      </c>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_deep_provenance_is_bounded_and_denied_without_recursion_failure</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>327</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>UT-327</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>test_v3_upgrade_is_explicit_additive_private_and_idempotent</t>
+        </is>
+      </c>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_v3_upgrade_is_explicit_additive_private_and_idempotent</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>328</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>UT-328</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>test_failure_after_classification_rolls_back_tables_rows_and_version</t>
+        </is>
+      </c>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_failure_after_classification_rolls_back_tables_rows_and_version</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>329</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>UT-329</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>test_scope_integrity_drift_is_rejected_without_repair</t>
+        </is>
+      </c>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_scope_integrity_drift_is_rejected_without_repair</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>330</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>UT-330</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>test_copy_preparation_reuses_backup_and_never_upgrades_source</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_copy_preparation_reuses_backup_and_never_upgrades_source</t>
+        </is>
+      </c>
+      <c r="K331" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>331</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>UT-331</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>test_failed_copy_keeps_verified_source_backup_and_original_data</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_failed_copy_keeps_verified_source_backup_and_original_data</t>
+        </is>
+      </c>
+      <c r="K332" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>332</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>UT-332</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>test_scope_copy_rejects_symlinks_existing_or_overlapping_destinations</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_scope_copy_rejects_symlinks_existing_or_overlapping_destinations</t>
+        </is>
+      </c>
+      <c r="K333" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>333</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>UT-333</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>test_precreated_scope_tables_do_not_authorize_automatic_v3_backfill</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_precreated_scope_tables_do_not_authorize_automatic_v3_backfill</t>
+        </is>
+      </c>
+      <c r="K334" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>334</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>UT-334</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>test_classification_replay_never_revives_revoked_sharing</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_classification_replay_never_revives_revoked_sharing</t>
+        </is>
+      </c>
+      <c r="K335" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>335</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>UT-335</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>test_revocation_from_another_session_invalidates_cached_grant</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_revocation_from_another_session_invalidates_cached_grant</t>
+        </is>
+      </c>
+      <c r="K336" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>336</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>UT-336</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>프로젝트·버전 공유·파생 출처</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>test_actual_source_owner_change_denies_stale_scope_metadata</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>tests/test_project_scopes.py::test_actual_source_owner_change_denies_stale_scope_metadata</t>
+        </is>
+      </c>
+      <c r="K337" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>337</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>UT-337</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>test_v4_copy_and_restore_preserve_revoked_grants_and_provenance</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_v4_copy_and_restore_preserve_revoked_grants_and_provenance</t>
+        </is>
+      </c>
+      <c r="K338" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>338</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>UT-338</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>test_v3_classification_isolated_for_two_owners_with_same_alias</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_v3_classification_isolated_for_two_owners_with_same_alias</t>
+        </is>
+      </c>
+      <c r="K339" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>339</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>UT-339</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>추가형 범위 이행·복제본·복구</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>test_populated_unversioned_complete_schema_requires_explicit_upgrade</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>tests/test_scope_migrations.py::test_populated_unversioned_complete_schema_requires_explicit_upgrade</t>
+        </is>
+      </c>
+      <c r="K340" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N313"/>
+  <autoFilter ref="A1:N340"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18388,7 +19927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18830,6 +20369,40 @@
       <c r="C26" t="inlineStr">
         <is>
           <t>자동 검증; 모델·운영 실행 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>REQ-PROJECT-SCOPE</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>개인 보관함/소유권/정확 버전 읽기 Grant/철회/파생 기억 출처 보존</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-MIGRATION</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>합성 v3→v4/원문 보존/재실행/실패 rollback/복제 DB·백업 복원/운영 미적용</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: P1-03 authenticated contract scope read gate
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$340</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$349</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>339개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>348개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N340"/>
+  <dimension ref="A1:N349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19915,8 +19915,521 @@
         </is>
       </c>
     </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>340</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>UT-340</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>test_owned_exact_read_and_permission_gate_adapter</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_owned_exact_read_and_permission_gate_adapter</t>
+        </is>
+      </c>
+      <c r="K341" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>341</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>UT-341</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>test_contract_cannot_enlarge_current_data_authority</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_contract_cannot_enlarge_current_data_authority</t>
+        </is>
+      </c>
+      <c r="K342" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>342</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>UT-342</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>test_claimed_actor_does_not_replace_authenticated_session</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_claimed_actor_does_not_replace_authenticated_session</t>
+        </is>
+      </c>
+      <c r="K343" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>343</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>UT-343</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>test_session_project_and_db_changes_fail_closed</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_session_project_and_db_changes_fail_closed</t>
+        </is>
+      </c>
+      <c r="K344" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>344</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>UT-344</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>test_read_grant_and_policy_generation_are_rechecked</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_read_grant_and_policy_generation_are_rechecked</t>
+        </is>
+      </c>
+      <c r="K345" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>345</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>UT-345</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>test_revoked_dependency_blocks_derived_memory_even_with_new_grant</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_revoked_dependency_blocks_derived_memory_even_with_new_grant</t>
+        </is>
+      </c>
+      <c r="K346" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>346</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>UT-346</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>test_gate_does_not_reclassify_or_write_content</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_gate_does_not_reclassify_or_write_content</t>
+        </is>
+      </c>
+      <c r="K347" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>347</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>UT-347</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>test_personal_inbox_is_explicit_and_not_a_project_wildcard</t>
+        </is>
+      </c>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_personal_inbox_is_explicit_and_not_a_project_wildcard</t>
+        </is>
+      </c>
+      <c r="K348" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>348</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>UT-348</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>인증 세션·계약·자료 권한 Gate</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>test_repository_reference_cannot_become_a_data_or_execution_capability</t>
+        </is>
+      </c>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>tests/test_scope_permissions.py::test_repository_reference_cannot_become_a_data_or_execution_capability</t>
+        </is>
+      </c>
+      <c r="K349" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N340"/>
+  <autoFilter ref="A1:N349"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
docs: complete scope permission QA coverage and verification record
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -20440,7 +20440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20914,6 +20914,23 @@
         </is>
       </c>
       <c r="C28" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>REQ-SCOPE-PERMISSION</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>인증 세션/소유권/정확 버전/정책 세대/철회/파생 출처 읽기 Gate, 실행 권한 확대 금지</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P1-04 scoped data paths, immutable archival and approved client protocol
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$349</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$368</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>348개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>367개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N349"/>
+  <dimension ref="A1:N368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20428,8 +20428,1091 @@
         </is>
       </c>
     </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>349</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>UT-349</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>현재 범위 읽기 Adapter</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>test_bridge_defaults_to_private_inbox_and_never_all_projects</t>
+        </is>
+      </c>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>tests/test_scoped_reads.py::test_bridge_defaults_to_private_inbox_and_never_all_projects</t>
+        </is>
+      </c>
+      <c r="K350" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>UT-350</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>현재 범위 읽기 Adapter</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>test_bridge_uses_current_grant_without_copying_source</t>
+        </is>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>tests/test_scoped_reads.py::test_bridge_uses_current_grant_without_copying_source</t>
+        </is>
+      </c>
+      <c r="K351" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>351</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>UT-351</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>현재 범위 읽기 Adapter</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>test_bridge_refuses_other_user_and_unknown_source_kind</t>
+        </is>
+      </c>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>tests/test_scoped_reads.py::test_bridge_refuses_other_user_and_unknown_source_kind</t>
+        </is>
+      </c>
+      <c r="K352" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>352</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>UT-352</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>현재 범위 읽기 Adapter</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>test_bridge_listing_never_autoflushes_uncommitted_changes</t>
+        </is>
+      </c>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I353" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J353" t="inlineStr">
+        <is>
+          <t>tests/test_scoped_reads.py::test_bridge_listing_never_autoflushes_uncommitted_changes</t>
+        </is>
+      </c>
+      <c r="K353" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>353</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>UT-353</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>test_data_routes_default_private_and_only_exact_grants_cross_projects</t>
+        </is>
+      </c>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I354" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J354" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_data_routes_default_private_and_only_exact_grants_cross_projects</t>
+        </is>
+      </c>
+      <c r="K354" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>354</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>UT-354</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>test_archival_preserves_original_chunks_versions_and_is_idempotent</t>
+        </is>
+      </c>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J355" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_archival_preserves_original_chunks_versions_and_is_idempotent</t>
+        </is>
+      </c>
+      <c r="K355" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>355</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>UT-355</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>test_memory_archival_preserves_history_and_hides_model_profile</t>
+        </is>
+      </c>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J356" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_memory_archival_preserves_history_and_hides_model_profile</t>
+        </is>
+      </c>
+      <c r="K356" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>356</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>UT-356</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>test_new_conversation_fixed_scope_legacy_conversation_never_auto_moved</t>
+        </is>
+      </c>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J357" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_new_conversation_fixed_scope_legacy_conversation_never_auto_moved</t>
+        </is>
+      </c>
+      <c r="K357" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>357</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>UT-357</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>test_grant_revoke_blocks_old_history_and_model_calls</t>
+        </is>
+      </c>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I358" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J358" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_grant_revoke_blocks_old_history_and_model_calls</t>
+        </is>
+      </c>
+      <c r="K358" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>358</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>UT-358</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>test_semantic_filters_before_embedding_and_rechecks_after_inference</t>
+        </is>
+      </c>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I359" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J359" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_semantic_filters_before_embedding_and_rechecks_after_inference</t>
+        </is>
+      </c>
+      <c r="K359" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>359</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>UT-359</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>test_extraction_ignores_model_project_and_rejects_legacy_before_model</t>
+        </is>
+      </c>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I360" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J360" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_extraction_ignores_model_project_and_rejects_legacy_before_model</t>
+        </is>
+      </c>
+      <c r="K360" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>UT-360</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>test_archive_backup_restore_keeps_tombstone_and_original</t>
+        </is>
+      </c>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I361" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J361" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_archive_backup_restore_keeps_tombstone_and_original</t>
+        </is>
+      </c>
+      <c r="K361" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>361</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>UT-361</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>test_archive_in_native_project_cannot_be_used_as_cross_project_delete_oracle</t>
+        </is>
+      </c>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I362" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J362" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_archive_in_native_project_cannot_be_used_as_cross_project_delete_oracle</t>
+        </is>
+      </c>
+      <c r="K362" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>362</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>UT-362</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>test_chat_drops_result_if_grant_revoked_while_model_is_running</t>
+        </is>
+      </c>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I363" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J363" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_chat_drops_result_if_grant_revoked_while_model_is_running</t>
+        </is>
+      </c>
+      <c r="K363" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>363</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>UT-363</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F364" t="inlineStr">
+        <is>
+          <t>test_other_user_and_missing_csrf_cannot_grant_or_archive</t>
+        </is>
+      </c>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I364" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J364" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_other_user_and_missing_csrf_cannot_grant_or_archive</t>
+        </is>
+      </c>
+      <c r="K364" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>364</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>UT-364</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>v5 추가형 이행·원문 보존</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F365" t="inlineStr">
+        <is>
+          <t>test_v5_adds_only_empty_boundary_tables_and_preserves_v4</t>
+        </is>
+      </c>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I365" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J365" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_migrations.py::test_v5_adds_only_empty_boundary_tables_and_preserves_v4</t>
+        </is>
+      </c>
+      <c r="K365" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>365</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>UT-365</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>v5 추가형 이행·원문 보존</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F366" t="inlineStr">
+        <is>
+          <t>test_v5_failure_rolls_back_new_ddl_and_version_without_losing_v4</t>
+        </is>
+      </c>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I366" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J366" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_migrations.py::test_v5_failure_rolls_back_new_ddl_and_version_without_losing_v4</t>
+        </is>
+      </c>
+      <c r="K366" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>UT-366</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>v5 추가형 이행·원문 보존</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F367" t="inlineStr">
+        <is>
+          <t>test_v5_integrity_drift_is_denied_without_repair</t>
+        </is>
+      </c>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I367" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J367" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_migrations.py::test_v5_integrity_drift_is_denied_without_repair</t>
+        </is>
+      </c>
+      <c r="K367" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>367</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>UT-367</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>문서·기억·대화·보관 경로</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F368" t="inlineStr">
+        <is>
+          <t>test_conversation_metadata_roundtrips_exact_project_and_stale_state</t>
+        </is>
+      </c>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I368" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J368" t="inlineStr">
+        <is>
+          <t>tests/test_scope_data_paths.py::test_conversation_metadata_roundtrips_exact_project_and_stale_state</t>
+        </is>
+      </c>
+      <c r="K368" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N349"/>
+  <autoFilter ref="A1:N368"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20440,7 +21523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20931,6 +22014,23 @@
         </is>
       </c>
       <c r="C29" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>REQ-SCOPED-DATA</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>개인 기본 격리/명시 버전 공유/보관/대화 고정/출처 추적/v5 보존·복구</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P1-05 live task approval and bounded tool enforcement
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$368</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$383</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>367개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>382개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N368"/>
+  <dimension ref="A1:N383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21511,8 +21511,863 @@
         </is>
       </c>
     </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>368</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>UT-368</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F369" t="inlineStr">
+        <is>
+          <t>test_contract_reference_alone_is_not_authority</t>
+        </is>
+      </c>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I369" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J369" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_contract_reference_alone_is_not_authority</t>
+        </is>
+      </c>
+      <c r="K369" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>369</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>UT-369</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F370" t="inlineStr">
+        <is>
+          <t>test_current_approval_is_bound_and_invalidated</t>
+        </is>
+      </c>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I370" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J370" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_current_approval_is_bound_and_invalidated</t>
+        </is>
+      </c>
+      <c r="K370" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>370</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>UT-370</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F371" t="inlineStr">
+        <is>
+          <t>test_logout_preserves_approval_history_but_blocks_use</t>
+        </is>
+      </c>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I371" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J371" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_logout_preserves_approval_history_but_blocks_use</t>
+        </is>
+      </c>
+      <c r="K371" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>371</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>UT-371</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F372" t="inlineStr">
+        <is>
+          <t>test_approval_evidence_is_immutable</t>
+        </is>
+      </c>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I372" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J372" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_approval_evidence_is_immutable</t>
+        </is>
+      </c>
+      <c r="K372" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>372</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>UT-372</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F373" t="inlineStr">
+        <is>
+          <t>test_revoked_reference_cannot_be_resurrected</t>
+        </is>
+      </c>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I373" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J373" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_revoked_reference_cannot_be_resurrected</t>
+        </is>
+      </c>
+      <c r="K373" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>373</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>UT-373</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F374" t="inlineStr">
+        <is>
+          <t>test_unknown_tools_never_reach_executor</t>
+        </is>
+      </c>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I374" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J374" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_unknown_tools_never_reach_executor</t>
+        </is>
+      </c>
+      <c r="K374" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>374</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>UT-374</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F375" t="inlineStr">
+        <is>
+          <t>test_session_keys_separate_projects_and_policy_generations</t>
+        </is>
+      </c>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I375" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J375" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_session_keys_separate_projects_and_policy_generations</t>
+        </is>
+      </c>
+      <c r="K375" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>375</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>UT-375</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F376" t="inlineStr">
+        <is>
+          <t>test_coding_read_and_propose_preserve_original</t>
+        </is>
+      </c>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I376" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J376" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_coding_read_and_propose_preserve_original</t>
+        </is>
+      </c>
+      <c r="K376" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>376</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>UT-376</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F377" t="inlineStr">
+        <is>
+          <t>test_revocation_during_registered_execution_discards_result</t>
+        </is>
+      </c>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I377" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J377" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_revocation_during_registered_execution_discards_result</t>
+        </is>
+      </c>
+      <c r="K377" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>377</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>UT-377</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F378" t="inlineStr">
+        <is>
+          <t>test_model_cannot_propose_security_or_test_edits</t>
+        </is>
+      </c>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I378" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J378" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_model_cannot_propose_security_or_test_edits</t>
+        </is>
+      </c>
+      <c r="K378" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>378</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>UT-378</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F379" t="inlineStr">
+        <is>
+          <t>test_http_approval_uses_auth_csrf_and_private_receipts</t>
+        </is>
+      </c>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I379" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J379" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_http_approval_uses_auth_csrf_and_private_receipts</t>
+        </is>
+      </c>
+      <c r="K379" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>379</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>UT-379</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>v6 승인 기록·보존·복구</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t>test_v6_requires_explicit_upgrade_preserves_and_repeats</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J380" t="inlineStr">
+        <is>
+          <t>tests/test_task_approval_migrations.py::test_v6_requires_explicit_upgrade_preserves_and_repeats</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>UT-380</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>v6 승인 기록·보존·복구</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t>test_v6_failed_guard_validation_rolls_back_all_new_ddl</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J381" t="inlineStr">
+        <is>
+          <t>tests/test_task_approval_migrations.py::test_v6_failed_guard_validation_rolls_back_all_new_ddl</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>381</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>UT-381</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>v6 승인 기록·보존·복구</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t>test_v6_guard_drift_never_auto_repairs</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J382" t="inlineStr">
+        <is>
+          <t>tests/test_task_approval_migrations.py::test_v6_guard_drift_never_auto_repairs</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>382</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>UT-382</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>v6 승인 기록·보존·복구</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t>test_v5_backup_restores_to_separate_inactive_destination</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J383" t="inlineStr">
+        <is>
+          <t>tests/test_task_approval_migrations.py::test_v5_backup_restores_to_separate_inactive_destination</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N368"/>
+  <autoFilter ref="A1:N383"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21523,7 +22378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22031,6 +22886,23 @@
         </is>
       </c>
       <c r="C30" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>인증·CSRF/계약 digest/세션·정책·도구 설정 바인딩/철회/경로 보호/v6 추가형 이행·복구</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
fix: bind tools to current role capabilities and portable test imports
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$383</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$384</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>382개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>383개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N383"/>
+  <dimension ref="A1:N384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22366,8 +22366,65 @@
         </is>
       </c>
     </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>383</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>UT-383</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t>test_role_capability_removed_blocks_new_approval</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J384" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_role_capability_removed_blocks_new_approval</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N383"/>
+  <autoFilter ref="A1:N384"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix: reject stale approval snapshots while preserving uncommitted data
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$384</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$386</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>383개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>385개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N384"/>
+  <dimension ref="A1:N386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22423,8 +22423,122 @@
         </is>
       </c>
     </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>384</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>UT-384</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t>test_explicit_wal_read_snapshot_cannot_reuse_revoked_approval</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J385" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_explicit_wal_read_snapshot_cannot_reuse_revoked_approval</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>385</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>UT-385</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>REQ-TASK-APPROVAL</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>유효 승인·도구 범위·계약 바인딩</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t>test_gate_rejects_flushed_writes_without_rolling_back_them</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J386" t="inlineStr">
+        <is>
+          <t>tests/test_task_approvals.py::test_gate_rejects_flushed_writes_without_rolling_back_them</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N384"/>
+  <autoFilter ref="A1:N386"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: P1-06 authenticated task lifecycle and atomic recoverable checkpoints
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$386</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$403</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>385개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>402개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N386"/>
+  <dimension ref="A1:N403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22537,8 +22537,977 @@
         </is>
       </c>
     </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>386</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>UT-386</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t>test_create_is_idempotent_but_contract_identity_is_not_replaceable</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J387" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_create_is_idempotent_but_contract_identity_is_not_replaceable</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>387</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>UT-387</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t>test_state_queue_requires_actual_approval_and_owner</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J388" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_state_queue_requires_actual_approval_and_owner</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>388</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>UT-388</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t>test_proposal_cannot_skip_state_machine_or_fake_success</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J389" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_proposal_cannot_skip_state_machine_or_fake_success</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>389</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>UT-389</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t>test_claim_lock_prevents_duplicate_worker_and_crash_requires_resume</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J390" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_claim_lock_prevents_duplicate_worker_and_crash_requires_resume</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>390</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>UT-390</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>test_persisted_running_checkpoint_is_never_automatically_replayed</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J391" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_persisted_running_checkpoint_is_never_automatically_replayed</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>391</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>UT-391</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>test_pause_resume_and_sticky_cancel</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J392" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_pause_resume_and_sticky_cancel</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>392</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>UT-392</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>test_only_current_approval_and_independent_verification_can_complete</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J393" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_only_current_approval_and_independent_verification_can_complete</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>393</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>UT-393</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>test_revocation_blocks_resume_and_does_not_rewrite_checkpoint</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J394" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_revocation_blocks_resume_and_does_not_rewrite_checkpoint</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>394</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>UT-394</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>test_corrupt_or_retargeted_checkpoint_fails_without_repair</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J395" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_corrupt_or_retargeted_checkpoint_fails_without_repair</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>395</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>UT-395</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>test_atomic_save_failure_preserves_previous_checkpoint</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J396" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_atomic_save_failure_preserves_previous_checkpoint</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>396</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>UT-396</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>test_restart_reads_same_contract_and_revision_without_executing</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J397" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_restart_reads_same_contract_and_revision_without_executing</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>397</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>UT-397</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>test_waiting_for_approval_and_early_pause_are_observations_only</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J398" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_waiting_for_approval_and_early_pause_are_observations_only</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>398</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>UT-398</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>test_cancel_during_verification_cannot_become_success</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J399" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_cancel_during_verification_cannot_become_success</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>399</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>UT-399</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>test_checkpoint_checksums_and_status_never_replace_db_approval</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J400" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_checkpoint_checksums_and_status_never_replace_db_approval</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>UT-400</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>test_http_state_endpoints_cannot_supply_arbitrary_completion</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J401" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_http_state_endpoints_cannot_supply_arbitrary_completion</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>401</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>UT-401</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>test_api_queue_requires_second_explicit_resume_after_crash</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J402" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_api_queue_requires_second_explicit_resume_after_crash</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>402</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>UT-402</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>상태 전이·체크포인트·중복 실행·재개</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>test_http_create_approve_queue_pause_resume_and_cancel</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J403" t="inlineStr">
+        <is>
+          <t>tests/test_task_checkpoints.py::test_http_create_approve_queue_pause_resume_and_cancel</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N386"/>
+  <autoFilter ref="A1:N403"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22549,7 +23518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23074,6 +24043,23 @@
         </is>
       </c>
       <c r="C31" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>REQ-TASK-STATE</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>불변 계약·실행 상태 분리/원자 체크포인트/소유권·CAS·lock/중단·재개/독립 검증</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P1-07 durable resource reservations and bounded recovery
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$403</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$418</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>402개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>417개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N403"/>
+  <dimension ref="A1:N418"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23506,8 +23506,863 @@
         </is>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>UT-403</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>test_measured_usage_refunds_reservation_and_duplicate_operation_never_replays</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J404" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_measured_usage_refunds_reservation_and_duplicate_operation_never_replays</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>404</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>UT-404</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>test_unmeasured_usage_preserves_reservation_and_is_not_reported_as_zero</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J405" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_unmeasured_usage_preserves_reservation_and_is_not_reported_as_zero</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>405</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>UT-405</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>test_known_busy_retries_are_bounded_and_charge_every_attempt</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J406" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_known_busy_retries_are_bounded_and_charge_every_attempt</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>406</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>UT-406</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>test_scope_or_unknown_failures_never_automatically_retry</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J407" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_scope_or_unknown_failures_never_automatically_retry</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>407</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>UT-407</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>test_token_budget_is_checked_before_callback</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J408" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_token_budget_is_checked_before_callback</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>UT-408</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>test_missing_or_overcommitted_vram_never_starts_callback</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J409" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_missing_or_overcommitted_vram_never_starts_callback</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>409</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>UT-409</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>test_gpu_admission_reuses_conservative_existing_math_without_policy_write</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J410" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_gpu_admission_reuses_conservative_existing_math_without_policy_write</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>410</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>UT-410</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>test_gpu_overrun_discards_result_instead_of_reporting_success</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J411" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_gpu_overrun_discards_result_instead_of_reporting_success</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>411</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>UT-411</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>test_revocation_after_operation_discards_value_and_stops</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J412" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_revocation_after_operation_discards_value_and_stops</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>412</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>UT-412</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>test_pending_intent_requires_explicit_recovery_and_never_refunds_unknown_call</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J413" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_pending_intent_requires_explicit_recovery_and_never_refunds_unknown_call</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>413</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>UT-413</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>test_cancelled_await_is_preserved_and_no_automatic_retry</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_cancelled_await_is_preserved_and_no_automatic_retry</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>414</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>UT-414</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>test_step_budget_cannot_be_reset_by_new_operation_ids</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J415" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_step_budget_cannot_be_reset_by_new_operation_ids</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>415</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>UT-415</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>test_expired_task_deadline_blocks_before_callback</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J416" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_expired_task_deadline_blocks_before_callback</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>416</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>UT-416</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>test_timed_out_operation_is_cancelled_charged_and_not_retried</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J417" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_timed_out_operation_is_cancelled_charged_and_not_retried</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>417</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>UT-417</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>제한 재시도·예약 ledger·시간/GPU·복구</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>test_runtime_checkpoint_corruption_never_resets_budget</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J418" t="inlineStr">
+        <is>
+          <t>tests/test_task_resources.py::test_runtime_checkpoint_corruption_never_resets_budget</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N403"/>
+  <autoFilter ref="A1:N418"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23518,7 +24373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24060,6 +24915,23 @@
         </is>
       </c>
       <c r="C32" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>REQ-TASK-RESOURCES</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>실패 분류·제한 재시도/단계·시간·토큰 예약/GPU admission/미측정 분리/중단 복구·무재실행</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P1-08 phase integration and offline task checkpoint companion backup
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$418</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$431</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>417개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>430개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N418"/>
+  <dimension ref="A1:N431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24361,8 +24361,749 @@
         </is>
       </c>
     </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>418</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>UT-418</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>test_full_phase_one_contract_gate_tool_runtime_independent_assertion_and_completion</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J419" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_full_phase_one_contract_gate_tool_runtime_independent_assertion_and_completion</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>419</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>UT-419</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>test_prompt_text_and_approval_id_cannot_grant_another_tool</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J420" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_prompt_text_and_approval_id_cannot_grant_another_tool</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>420</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>UT-420</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>test_same_user_cross_project_read_requires_exact_current_grant_and_revoke_blocks_runtime</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J421" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_same_user_cross_project_read_requires_exact_current_grant_and_revoke_blocks_runtime</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>421</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>UT-421</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>test_other_user_cannot_create_a_checkpoint_for_existing_contract</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J422" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_other_user_cannot_create_a_checkpoint_for_existing_contract</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>422</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>UT-422</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>test_offline_companion_restores_rows_and_pending_checkpoints_inactive_without_replay</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J423" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_offline_companion_restores_rows_and_pending_checkpoints_inactive_without_replay</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>423</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>UT-423</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>test_active_execution_lease_prevents_companion_backup_and_preserves_source</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J424" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_active_execution_lease_prevents_companion_backup_and_preserves_source</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>424</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>UT-424</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t>test_companion_corruption_is_rejected_without_overwriting_restore_target</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_companion_corruption_is_rejected_without_overwriting_restore_target</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>425</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>UT-425</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t>test_companion_requires_offline_and_new_nonoverlapping_destinations</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_companion_requires_offline_and_new_nonoverlapping_destinations</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>426</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>UT-426</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t>test_backup_and_gpu_policy_code_are_model_read_only</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_backup_and_gpu_policy_code_are_model_read_only</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>427</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>UT-427</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t>test_companion_preserves_revoked_grants_and_approval_tombstones</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_companion_preserves_revoked_grants_and_approval_tombstones</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>428</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>UT-428</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t>test_state_root_change_invalidates_old_approval_instead_of_resetting_budget</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J429" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_state_root_change_invalidates_old_approval_instead_of_resetting_budget</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>429</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>UT-429</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t>test_companion_empty_task_root_does_not_create_original_job_directory</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J430" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_companion_empty_task_root_does_not_create_original_job_directory</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>430</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>UT-430</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>공통 계약·격리·승인·복구 통합</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t>test_companion_detects_a_writer_ignoring_offline_locks_without_repairing_source</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J431" t="inlineStr">
+        <is>
+          <t>tests/test_phase_one_integration.py::test_companion_detects_a_writer_ignoring_offline_locks_without_repairing_source</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N418"/>
+  <autoFilter ref="A1:N431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24373,7 +25114,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24932,6 +25673,23 @@
         </is>
       </c>
       <c r="C33" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>REQ-PHASE-ONE-INTEGRATION</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>P1-01~07/승인 우회·철회·소유권/원본 보존/DB+공통 checkpoint 비활성 복원</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P2-A select audited checkpoint diagnostics without benchmark side effects
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$431</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$437</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>430개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>436개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N431"/>
+  <dimension ref="A1:N437"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25102,8 +25102,350 @@
         </is>
       </c>
     </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>431</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>UT-431</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t>test_checkpoint_write_error_survives_file_lock_and_keeps_previous_revision</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J432" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_checkpoint_write_error_survives_file_lock_and_keeps_previous_revision</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>432</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>UT-432</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t>test_suppressed_permission_cause_is_bounded_and_message_free</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J433" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_suppressed_permission_cause_is_bounded_and_message_free</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>433</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>UT-433</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t>test_selected_diagnostics_do_not_become_execution_authority</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J434" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_selected_diagnostics_do_not_become_execution_authority</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>434</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>UT-434</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t>test_automatic_tests_and_context_overrides_are_not_imported</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J435" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_automatic_tests_and_context_overrides_are_not_imported</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>435</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>UT-435</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t>test_runtime_storage_failure_does_not_replay_or_start_callback</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J436" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_runtime_storage_failure_does_not_replay_or_start_callback</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>436</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>UT-436</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>검증된 PR30 기반·PR31 오류/체크포인트 선별</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t>test_coding_control_reports_storage_failure_without_success_or_private_text</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J437" t="inlineStr">
+        <is>
+          <t>tests/test_evaluation_reuse.py::test_coding_control_reports_storage_failure_without_success_or_private_text</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N431"/>
+  <autoFilter ref="A1:N437"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25114,7 +25456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25690,6 +26032,23 @@
         </is>
       </c>
       <c r="C34" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>REQ-EVALUATION-REUSE</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PR30 현재 기반 재사용/PR31 typed checkpoint 오류·bounded type-only 분류/저장 보존/HostRunner·자동테스트 미도입</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: P2-B synthetic tasks and independent offline oracle grading
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$437</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$446</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>436개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>445개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N437"/>
+  <dimension ref="A1:N446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25444,8 +25444,521 @@
         </is>
       </c>
     </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>437</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>UT-437</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t>test_ten_mixed_tasks_are_reproducible_and_public_view_excludes_oracle</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J438" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_ten_mixed_tasks_are_reproducible_and_public_view_excludes_oracle</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>438</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>UT-438</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t>test_external_oracle_compares_all_cases_without_accepting_model_scores</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J439" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_external_oracle_compares_all_cases_without_accepting_model_scores</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>439</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>UT-439</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t>test_fake_scores_missing_evidence_or_failure_cannot_be_success</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J440" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_fake_scores_missing_evidence_or_failure_cannot_be_success</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>440</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>UT-440</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t>test_seed_or_task_or_path_cannot_be_changed_after_approval</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J441" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_seed_or_task_or_path_cannot_be_changed_after_approval</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>UT-441</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t>test_revocation_while_runner_executes_retains_audit_but_blocks_result</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J442" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_revocation_while_runner_executes_retains_audit_but_blocks_result</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>442</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>UT-442</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t>test_cleanup_uncertainty_blocks_next_runner_without_auto_recovery</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J443" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_cleanup_uncertainty_blocks_next_runner_without_auto_recovery</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>443</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>UT-443</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t>test_input_mutation_and_numeric_type_changes_are_detected</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J444" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_input_mutation_and_numeric_type_changes_are_detected</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>444</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>UT-444</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t>test_real_grader_rejects_nonisolated_application_image_before_execution</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J445" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_real_grader_rejects_nonisolated_application_image_before_execution</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>445</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>UT-445</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t>test_oracle_public_answers_match_independent_spec_examples</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J446" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_oracle_public_answers_match_independent_spec_examples</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N437"/>
+  <autoFilter ref="A1:N446"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25456,7 +25969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26049,6 +26562,23 @@
         </is>
       </c>
       <c r="C35" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>합성 Role-AI5/소형5·공개2/숨김4/정답 외부 채점·위조/철회/cleanup 차단·로컬 보고서</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
fix: decode one grader vector across mixed unittest output without accepting duplicates
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$446</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$447</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>445개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>446개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N446"/>
+  <dimension ref="A1:N447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25957,8 +25957,65 @@
         </is>
       </c>
     </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>446</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>UT-446</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>REQ-INDEPENDENT-GRADING</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>혼합10과제·공개/숨김·외부 oracle·증거 보존</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t>test_combined_unittest_progress_does_not_hide_or_duplicate_machine_evidence</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J447" t="inlineStr">
+        <is>
+          <t>tests/test_independent_evaluation.py::test_combined_unittest_progress_does_not_hide_or_duplicate_machine_evidence</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N446"/>
+  <autoFilter ref="A1:N447"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: bind local coding delegation to common task execution
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$447</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$458</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>446개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>457개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N447"/>
+  <dimension ref="A1:N458"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26014,8 +26014,635 @@
         </is>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>447</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>UT-447</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t>test_common_pipeline_requires_independent_success_and_preserves_source</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J448" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_common_pipeline_requires_independent_success_and_preserves_source</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>448</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>UT-448</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t>test_public_success_cannot_override_hidden_failure</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J449" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_public_success_cannot_override_hidden_failure</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>449</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>UT-449</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t>test_unknown_tokens_remain_unmeasured_and_reserved</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J450" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_unknown_tokens_remain_unmeasured_and_reserved</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>450</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>UT-450</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t>test_model_cannot_write_tests_or_escape_exact_contract</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J451" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_model_cannot_write_tests_or_escape_exact_contract</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>451</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>UT-451</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t>test_cancel_after_model_discards_output_before_patch</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J452" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_cancel_after_model_discards_output_before_patch</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>452</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>UT-452</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t>test_revocation_during_independent_grading_prevents_completion</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J453" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_revocation_during_independent_grading_prevents_completion</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>453</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>UT-453</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E454" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t>test_missing_current_approval_never_creates_legacy_job</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J454" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_missing_current_approval_never_creates_legacy_job</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>454</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>UT-454</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>공통 계약·기존 Coding Agent·독립 채점 연결</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t>test_no_hidden_grading_or_success_when_step_budget_exhausts</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J455" t="inlineStr">
+        <is>
+          <t>tests/test_task_delegation.py::test_no_hidden_grading_or_success_when_step_budget_exhausts</t>
+        </is>
+      </c>
+      <c r="K455" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>455</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>UT-455</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>REQ-WINDOWS-LOOPBACK</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>고정 Windows loopback·무권한 데이터 전달</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F456" t="inlineStr">
+        <is>
+          <t>test_untrusted_model_message_never_becomes_powershell_source_or_credentials</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J456" t="inlineStr">
+        <is>
+          <t>tests/test_windows_loopback_transport.py::test_untrusted_model_message_never_becomes_powershell_source_or_credentials</t>
+        </is>
+      </c>
+      <c r="K456" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>456</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>UT-456</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>REQ-WINDOWS-LOOPBACK</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>고정 Windows loopback·무권한 데이터 전달</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t>test_unsupported_network_model_or_cache_operations_never_execute</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J457" t="inlineStr">
+        <is>
+          <t>tests/test_windows_loopback_transport.py::test_unsupported_network_model_or_cache_operations_never_execute</t>
+        </is>
+      </c>
+      <c r="K457" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>457</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>UT-457</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>REQ-WINDOWS-LOOPBACK</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>고정 Windows loopback·무권한 데이터 전달</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F458" t="inlineStr">
+        <is>
+          <t>test_transport_does_not_follow_redirects_or_copy_private_failure_text</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J458" t="inlineStr">
+        <is>
+          <t>tests/test_windows_loopback_transport.py::test_transport_does_not_follow_redirects_or_copy_private_failure_text</t>
+        </is>
+      </c>
+      <c r="K458" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N447"/>
+  <autoFilter ref="A1:N458"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26026,7 +26653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26636,6 +27263,40 @@
         </is>
       </c>
       <c r="C36" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>REQ-TASK-DELEGATION</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>기존 Coding Agent/common gate·예산 ledger/공개·독립 채점 분리·취소/철회 차단</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>REQ-WINDOWS-LOOPBACK</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>고정 localhost11434/상수 PowerShell·stdin 데이터/설치·원격·generate 차단</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: qualify evaluation metrics and preserve unknown evidence
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$458</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$466</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>457개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>465개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N458"/>
+  <dimension ref="A1:N466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26641,8 +26641,464 @@
         </is>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>458</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>UT-458</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F459" t="inlineStr">
+        <is>
+          <t>test_unknown_tokens_and_missing_scores_never_become_zero_or_success</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J459" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_unknown_tokens_and_missing_scores_never_become_zero_or_success</t>
+        </is>
+      </c>
+      <c r="K459" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>459</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>UT-459</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F460" t="inlineStr">
+        <is>
+          <t>test_synthetic_runs_cannot_inflate_actual_performance_and_duplicates_rejected</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J460" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_synthetic_runs_cannot_inflate_actual_performance_and_duplicates_rejected</t>
+        </is>
+      </c>
+      <c r="K460" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>460</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>UT-460</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F461" t="inlineStr">
+        <is>
+          <t>test_invalid_or_unproven_measurements_are_rejected</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J461" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_invalid_or_unproven_measurements_are_rejected</t>
+        </is>
+      </c>
+      <c r="K461" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>461</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>UT-461</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F462" t="inlineStr">
+        <is>
+          <t>test_observer_keeps_numeric_samples_and_labels_device_wide_peak</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J462" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_observer_keeps_numeric_samples_and_labels_device_wide_peak</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>462</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>UT-462</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t>test_missing_or_bad_gpu_measurements_preserve_null_and_error_counts</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J463" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_missing_or_bad_gpu_measurements_preserve_null_and_error_counts</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>463</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>UT-463</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t>test_sampling_capacity_is_bounded_and_partial_coverage_not_complete</t>
+        </is>
+      </c>
+      <c r="G464" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H464" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I464" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J464" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_sampling_capacity_is_bounded_and_partial_coverage_not_complete</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>464</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>UT-464</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t>test_recovery_denominator_counts_attempted_runs_and_preserves_failures</t>
+        </is>
+      </c>
+      <c r="G465" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H465" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I465" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J465" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_recovery_denominator_counts_attempted_runs_and_preserves_failures</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>465</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>UT-465</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>실측/미측정·실패 분모·GPU 샘플·증거 보존</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t>test_measured_pipeline_receipt_and_second_attempt_preserve_previous_evidence</t>
+        </is>
+      </c>
+      <c r="G466" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H466" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I466" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J466" t="inlineStr">
+        <is>
+          <t>tests/test_task_metrics.py::test_measured_pipeline_receipt_and_second_attempt_preserve_previous_evidence</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N458"/>
+  <autoFilter ref="A1:N466"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26653,7 +27109,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27297,6 +27753,23 @@
         </is>
       </c>
       <c r="C38" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>REQ-TASK-METRICS</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>실제/합성 구분·토큰 null·GPU 관측·미채점 분모·실행 중복 보존</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: prepare conservative paired evaluation and public baseline workflow
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$466</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$480</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>465개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>479개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N466"/>
+  <dimension ref="A1:N480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27097,8 +27097,806 @@
         </is>
       </c>
     </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>466</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>UT-466</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t>test_public_package_has_ten_goals_stubs_public_tests_and_no_hidden_source</t>
+        </is>
+      </c>
+      <c r="G467" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H467" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I467" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J467" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_public_package_has_ten_goals_stubs_public_tests_and_no_hidden_source</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>467</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>UT-467</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t>test_public_fixture_tampering_or_extra_sources_fail_closed</t>
+        </is>
+      </c>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_public_fixture_tampering_or_extra_sources_fail_closed</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>468</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>UT-468</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t>test_missing_real_data_cannot_be_called_complete_or_improved</t>
+        </is>
+      </c>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_missing_real_data_cannot_be_called_complete_or_improved</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>469</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>UT-469</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t>test_synthetic_records_are_excluded_even_when_scores_look_perfect</t>
+        </is>
+      </c>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_synthetic_records_are_excluded_even_when_scores_look_perfect</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>470</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>UT-470</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t>test_equal_quality_without_codex_usage_remains_inconclusive</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_equal_quality_without_codex_usage_remains_inconclusive</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>471</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>UT-471</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t>test_changed_tasks_conditions_or_code_are_not_comparable</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_changed_tasks_conditions_or_code_are_not_comparable</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>472</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>UT-472</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F473" t="inlineStr">
+        <is>
+          <t>test_lower_token_count_cannot_hide_quality_regression</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J473" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_lower_token_count_cannot_hide_quality_regression</t>
+        </is>
+      </c>
+      <c r="K473" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>473</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>UT-473</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E474" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F474" t="inlineStr">
+        <is>
+          <t>test_unequal_repeats_or_duplicate_runs_cannot_bias_comparison</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J474" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_unequal_repeats_or_duplicate_runs_cannot_bias_comparison</t>
+        </is>
+      </c>
+      <c r="K474" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>474</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>UT-474</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F475" t="inlineStr">
+        <is>
+          <t>test_actual_usage_still_requires_blind_protocol_and_all_six_ci_checks</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J475" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_actual_usage_still_requires_blind_protocol_and_all_six_ci_checks</t>
+        </is>
+      </c>
+      <c r="K475" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>475</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>UT-475</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E476" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F476" t="inlineStr">
+        <is>
+          <t>test_complete_synthetic_fixture_proves_logic_only_not_actual_performance</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J476" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_complete_synthetic_fixture_proves_logic_only_not_actual_performance</t>
+        </is>
+      </c>
+      <c r="K476" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>476</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>UT-476</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E477" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F477" t="inlineStr">
+        <is>
+          <t>test_direct_baseline_unknown_calls_time_and_recovery_remain_null</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J477" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_direct_baseline_unknown_calls_time_and_recovery_remain_null</t>
+        </is>
+      </c>
+      <c r="K477" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>477</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>UT-477</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E478" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F478" t="inlineStr">
+        <is>
+          <t>test_all_failed_delegations_never_count_as_token_improvement</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J478" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_all_failed_delegations_never_count_as_token_improvement</t>
+        </is>
+      </c>
+      <c r="K478" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>478</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>UT-478</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E479" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F479" t="inlineStr">
+        <is>
+          <t>test_cli_regression_has_nonzero_exit_even_when_receipts_parse</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J479" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_cli_regression_has_nonzero_exit_even_when_receipts_parse</t>
+        </is>
+      </c>
+      <c r="K479" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>479</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>UT-479</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>동일10과제·원문/조건 고정·비교/미측정·기준선</t>
+        </is>
+      </c>
+      <c r="E480" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F480" t="inlineStr">
+        <is>
+          <t>test_producer_receipt_cannot_be_reused_for_different_candidate</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J480" t="inlineStr">
+        <is>
+          <t>tests/test_task_comparison.py::test_producer_receipt_cannot_be_reused_for_different_candidate</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N466"/>
+  <autoFilter ref="A1:N480"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27109,7 +27907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27770,6 +28568,23 @@
         </is>
       </c>
       <c r="C39" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>REQ-TASK-COMPARISON</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>공개 기준선/독립 채점/버전·seed·조건/실제·합성/회귀 차단·불충분 보류</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
feat: bind benchmark evaluation to private rootless endpoints
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$480</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$487</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>479개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>486개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N480"/>
+  <dimension ref="A1:N487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27895,8 +27895,407 @@
         </is>
       </c>
     </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>480</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>UT-480</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t>test_private_socket_binding_is_explicit_and_never_changes_process_context</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J481" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_private_socket_binding_is_explicit_and_never_changes_process_context</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>481</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>UT-481</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E482" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
+        <is>
+          <t>test_noncanonical_remote_and_oversized_inputs_are_rejected</t>
+        </is>
+      </c>
+      <c r="G482" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H482" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I482" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J482" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_noncanonical_remote_and_oversized_inputs_are_rejected</t>
+        </is>
+      </c>
+      <c r="K482" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>482</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>UT-482</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E483" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F483" t="inlineStr">
+        <is>
+          <t>test_bad_socket_type_links_permissions_and_ownership_fail_closed</t>
+        </is>
+      </c>
+      <c r="G483" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H483" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I483" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J483" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_bad_socket_type_links_permissions_and_ownership_fail_closed</t>
+        </is>
+      </c>
+      <c r="K483" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>483</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>UT-483</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E484" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F484" t="inlineStr">
+        <is>
+          <t>test_replaced_socket_invalidates_existing_task_approval</t>
+        </is>
+      </c>
+      <c r="G484" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H484" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I484" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J484" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_replaced_socket_invalidates_existing_task_approval</t>
+        </is>
+      </c>
+      <c r="K484" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>484</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>UT-484</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E485" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F485" t="inlineStr">
+        <is>
+          <t>test_explicit_endpoint_requires_existing_resource_preflight</t>
+        </is>
+      </c>
+      <c r="G485" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H485" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I485" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J485" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_explicit_endpoint_requires_existing_resource_preflight</t>
+        </is>
+      </c>
+      <c r="K485" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>485</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>UT-485</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E486" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F486" t="inlineStr">
+        <is>
+          <t>test_delegation_cli_forwards_socket_before_any_model_call</t>
+        </is>
+      </c>
+      <c r="G486" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H486" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I486" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J486" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_delegation_cli_forwards_socket_before_any_model_call</t>
+        </is>
+      </c>
+      <c r="K486" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>486</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>UT-486</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>명시적 사용자 Unix socket·실시간 바인딩·자원 preflight</t>
+        </is>
+      </c>
+      <c r="E487" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F487" t="inlineStr">
+        <is>
+          <t>test_baseline_cli_forwards_same_explicit_socket</t>
+        </is>
+      </c>
+      <c r="G487" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H487" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I487" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J487" t="inlineStr">
+        <is>
+          <t>tests/test_task_runtime_endpoint.py::test_baseline_cli_forwards_same_explicit_socket</t>
+        </is>
+      </c>
+      <c r="K487" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N480"/>
+  <autoFilter ref="A1:N487"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27907,7 +28306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28585,6 +28984,23 @@
         </is>
       </c>
       <c r="C40" t="inlineStr">
+        <is>
+          <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>REQ-BENCHMARK-ENDPOINT</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>A/B 로컬 Unix socket 선택·소유권/링크/교체 거부·Rootless 자원 제한·기존 기본값 보존</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>자동 검증; 실제 모델·학습·운영 반영 없음</t>
         </is>

</xml_diff>

<commit_message>
fix: keep sandbox inputs readable under restrictive umask
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$487</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$488</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -453,7 +453,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>486개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
+          <t>487개 시나리오; 매개변수별 실행 수는 결과에 기록</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N487"/>
+  <dimension ref="A1:N488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28294,8 +28294,65 @@
         </is>
       </c>
     </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>UT-487</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>REQ-CODE-EXECUTION</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>umask·비root bind·호스트 부모 비공개</t>
+        </is>
+      </c>
+      <c r="E488" t="inlineStr">
+        <is>
+          <t>단위/API</t>
+        </is>
+      </c>
+      <c r="F488" t="inlineStr">
+        <is>
+          <t>test_runner_mount_readable_without_exposing_private_parent</t>
+        </is>
+      </c>
+      <c r="G488" t="inlineStr">
+        <is>
+          <t>합성 설정·임시 DB·로컬 fixture</t>
+        </is>
+      </c>
+      <c r="H488" t="inlineStr">
+        <is>
+          <t>설정·인증·격리·무변경 조건을 pytest로 검사</t>
+        </is>
+      </c>
+      <c r="I488" t="inlineStr">
+        <is>
+          <t>무권한 접근·실행 차단, 비밀 및 기존 상태 보존</t>
+        </is>
+      </c>
+      <c r="J488" t="inlineStr">
+        <is>
+          <t>tests/test_code_execution_permissions.py::test_runner_mount_readable_without_exposing_private_parent</t>
+        </is>
+      </c>
+      <c r="K488" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N487"/>
+  <autoFilter ref="A1:N488"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
test: register Ollama response scenarios in Excel plan
</commit_message>
<xml_diff>
--- a/qa/Role-AI_unit_tests.xlsx
+++ b/qa/Role-AI_unit_tests.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'요약'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$488</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'단위테스트'!$A$1:$N$490</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'요구사항커버리지'!$A$1:$C$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'실환경검증'!$A$1:$D$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'결함이력'!$A$1:$E$3</definedName>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N488"/>
+  <dimension ref="A1:N490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28351,8 +28351,122 @@
         </is>
       </c>
     </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>488</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>UT-488</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>REQ-PROVIDER-SEC</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>boundaries</t>
+        </is>
+      </c>
+      <c r="E489" t="inlineStr">
+        <is>
+          <t>단위·경계</t>
+        </is>
+      </c>
+      <c r="F489" t="inlineStr">
+        <is>
+          <t>test_ollama_rejects_invalid_content_even_with_thinking</t>
+        </is>
+      </c>
+      <c r="G489" t="inlineStr">
+        <is>
+          <t>임시 SQLite·테스트 계정·Mock HTTP/Trainer; 실제 키·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H489" t="inlineStr">
+        <is>
+          <t>Mock HTTP에 대화 요청</t>
+        </is>
+      </c>
+      <c r="I489" t="inlineStr">
+        <is>
+          <t>빈 값·공백·비문자열·길이 초과 content 거부, thinking 비공개</t>
+        </is>
+      </c>
+      <c r="J489" t="inlineStr">
+        <is>
+          <t>tests/test_boundaries.py::test_ollama_rejects_invalid_content_even_with_thinking</t>
+        </is>
+      </c>
+      <c r="K489" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>489</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>UT-489</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>REQ-PROVIDER-SEC</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>boundaries</t>
+        </is>
+      </c>
+      <c r="E490" t="inlineStr">
+        <is>
+          <t>단위·경계</t>
+        </is>
+      </c>
+      <c r="F490" t="inlineStr">
+        <is>
+          <t>test_ollama_thinking_only_reply_becomes_chat_503</t>
+        </is>
+      </c>
+      <c r="G490" t="inlineStr">
+        <is>
+          <t>임시 SQLite·테스트 계정·Mock HTTP/Trainer; 실제 키·GPU 불필요</t>
+        </is>
+      </c>
+      <c r="H490" t="inlineStr">
+        <is>
+          <t>Mock HTTP에 대화 요청</t>
+        </is>
+      </c>
+      <c r="I490" t="inlineStr">
+        <is>
+          <t>합성 thinking-only 응답의 채팅 503 및 이력 미저장</t>
+        </is>
+      </c>
+      <c r="J490" t="inlineStr">
+        <is>
+          <t>tests/test_boundaries.py::test_ollama_thinking_only_reply_becomes_chat_503</t>
+        </is>
+      </c>
+      <c r="K490" t="inlineStr">
+        <is>
+          <t>미실행</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N488"/>
+  <autoFilter ref="A1:N490"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>